<commit_message>
Fill FSSAI and Brand Names sheets from two outlet certificates
</commit_message>
<xml_diff>
--- a/Compliance_Management_Tracker.xlsx
+++ b/Compliance_Management_Tracker.xlsx
@@ -31,9 +31,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="DD-MMM-YYYY"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="DD-MMM-YYYY"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -151,7 +150,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -185,10 +184,16 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -880,7 +885,7 @@
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>Sample Brand A</t>
+          <t>JS Concepts &amp; Solutions Pvt Ltd</t>
         </is>
       </c>
       <c r="C2" s="14" t="inlineStr">
@@ -890,16 +895,16 @@
       </c>
       <c r="D2" s="14" t="inlineStr">
         <is>
-          <t>ABC Foods Pvt Ltd</t>
+          <t>JS Concepts &amp; Solutions Private Limited</t>
         </is>
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>TM-1234567</t>
-        </is>
-      </c>
-      <c r="F2" s="15" t="n">
-        <v>45823</v>
+          <t>FSSAI: 22726442000324</t>
+        </is>
+      </c>
+      <c r="F2" s="17" t="n">
+        <v>46151</v>
       </c>
       <c r="G2" s="14" t="inlineStr">
         <is>
@@ -908,7 +913,7 @@
       </c>
       <c r="H2" s="14" t="inlineStr">
         <is>
-          <t>Primary brand</t>
+          <t>Outlet 1 - Bennett University, TechZone II, Greater Noida, UP - 201310</t>
         </is>
       </c>
     </row>
@@ -918,33 +923,37 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>Sample Brand B</t>
+          <t>Parma Food &amp; Beverage</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>Cloud Kitchen</t>
+          <t>Food &amp; Beverage</t>
         </is>
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>ABC Foods Pvt Ltd</t>
+          <t>Jatin Jhawar</t>
         </is>
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>TM-7654321</t>
-        </is>
-      </c>
-      <c r="F3" s="16" t="n">
-        <v>46103</v>
+          <t>FSSAI: 22726442000472</t>
+        </is>
+      </c>
+      <c r="F3" s="18" t="n">
+        <v>46218</v>
       </c>
       <c r="G3" s="6" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="H3" s="6" t="inlineStr"/>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>Outlet 2 - Bennett University, TechZone 2, Greater Noida, UP - 201310</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="n"/>
@@ -952,7 +961,7 @@
       <c r="C4" s="14" t="n"/>
       <c r="D4" s="14" t="n"/>
       <c r="E4" s="14" t="n"/>
-      <c r="F4" s="15" t="n"/>
+      <c r="F4" s="17" t="n"/>
       <c r="G4" s="14" t="n"/>
       <c r="H4" s="14" t="n"/>
     </row>
@@ -962,7 +971,7 @@
       <c r="C5" s="6" t="n"/>
       <c r="D5" s="6" t="n"/>
       <c r="E5" s="6" t="n"/>
-      <c r="F5" s="16" t="n"/>
+      <c r="F5" s="18" t="n"/>
       <c r="G5" s="6" t="n"/>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -972,7 +981,7 @@
       <c r="C6" s="14" t="n"/>
       <c r="D6" s="14" t="n"/>
       <c r="E6" s="14" t="n"/>
-      <c r="F6" s="15" t="n"/>
+      <c r="F6" s="17" t="n"/>
       <c r="G6" s="14" t="n"/>
       <c r="H6" s="14" t="n"/>
     </row>
@@ -982,7 +991,7 @@
       <c r="C7" s="6" t="n"/>
       <c r="D7" s="6" t="n"/>
       <c r="E7" s="6" t="n"/>
-      <c r="F7" s="16" t="n"/>
+      <c r="F7" s="18" t="n"/>
       <c r="G7" s="6" t="n"/>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -992,7 +1001,7 @@
       <c r="C8" s="14" t="n"/>
       <c r="D8" s="14" t="n"/>
       <c r="E8" s="14" t="n"/>
-      <c r="F8" s="15" t="n"/>
+      <c r="F8" s="17" t="n"/>
       <c r="G8" s="14" t="n"/>
       <c r="H8" s="14" t="n"/>
     </row>
@@ -1002,7 +1011,7 @@
       <c r="C9" s="6" t="n"/>
       <c r="D9" s="6" t="n"/>
       <c r="E9" s="6" t="n"/>
-      <c r="F9" s="16" t="n"/>
+      <c r="F9" s="18" t="n"/>
       <c r="G9" s="6" t="n"/>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -1012,7 +1021,7 @@
       <c r="C10" s="14" t="n"/>
       <c r="D10" s="14" t="n"/>
       <c r="E10" s="14" t="n"/>
-      <c r="F10" s="15" t="n"/>
+      <c r="F10" s="17" t="n"/>
       <c r="G10" s="14" t="n"/>
       <c r="H10" s="14" t="n"/>
     </row>
@@ -1022,7 +1031,7 @@
       <c r="C11" s="6" t="n"/>
       <c r="D11" s="6" t="n"/>
       <c r="E11" s="6" t="n"/>
-      <c r="F11" s="16" t="n"/>
+      <c r="F11" s="18" t="n"/>
       <c r="G11" s="6" t="n"/>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -1032,7 +1041,7 @@
       <c r="C12" s="14" t="n"/>
       <c r="D12" s="14" t="n"/>
       <c r="E12" s="14" t="n"/>
-      <c r="F12" s="15" t="n"/>
+      <c r="F12" s="17" t="n"/>
       <c r="G12" s="14" t="n"/>
       <c r="H12" s="14" t="n"/>
     </row>
@@ -1042,7 +1051,7 @@
       <c r="C13" s="6" t="n"/>
       <c r="D13" s="6" t="n"/>
       <c r="E13" s="6" t="n"/>
-      <c r="F13" s="16" t="n"/>
+      <c r="F13" s="18" t="n"/>
       <c r="G13" s="6" t="n"/>
       <c r="H13" s="6" t="n"/>
     </row>
@@ -1052,7 +1061,7 @@
       <c r="C14" s="14" t="n"/>
       <c r="D14" s="14" t="n"/>
       <c r="E14" s="14" t="n"/>
-      <c r="F14" s="15" t="n"/>
+      <c r="F14" s="17" t="n"/>
       <c r="G14" s="14" t="n"/>
       <c r="H14" s="14" t="n"/>
     </row>
@@ -1062,7 +1071,7 @@
       <c r="C15" s="6" t="n"/>
       <c r="D15" s="6" t="n"/>
       <c r="E15" s="6" t="n"/>
-      <c r="F15" s="16" t="n"/>
+      <c r="F15" s="18" t="n"/>
       <c r="G15" s="6" t="n"/>
       <c r="H15" s="6" t="n"/>
     </row>
@@ -1072,7 +1081,7 @@
       <c r="C16" s="14" t="n"/>
       <c r="D16" s="14" t="n"/>
       <c r="E16" s="14" t="n"/>
-      <c r="F16" s="15" t="n"/>
+      <c r="F16" s="17" t="n"/>
       <c r="G16" s="14" t="n"/>
       <c r="H16" s="14" t="n"/>
     </row>
@@ -1082,7 +1091,7 @@
       <c r="C17" s="6" t="n"/>
       <c r="D17" s="6" t="n"/>
       <c r="E17" s="6" t="n"/>
-      <c r="F17" s="16" t="n"/>
+      <c r="F17" s="18" t="n"/>
       <c r="G17" s="6" t="n"/>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -1092,7 +1101,7 @@
       <c r="C18" s="14" t="n"/>
       <c r="D18" s="14" t="n"/>
       <c r="E18" s="14" t="n"/>
-      <c r="F18" s="15" t="n"/>
+      <c r="F18" s="17" t="n"/>
       <c r="G18" s="14" t="n"/>
       <c r="H18" s="14" t="n"/>
     </row>
@@ -1102,7 +1111,7 @@
       <c r="C19" s="6" t="n"/>
       <c r="D19" s="6" t="n"/>
       <c r="E19" s="6" t="n"/>
-      <c r="F19" s="16" t="n"/>
+      <c r="F19" s="18" t="n"/>
       <c r="G19" s="6" t="n"/>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -1112,7 +1121,7 @@
       <c r="C20" s="14" t="n"/>
       <c r="D20" s="14" t="n"/>
       <c r="E20" s="14" t="n"/>
-      <c r="F20" s="15" t="n"/>
+      <c r="F20" s="17" t="n"/>
       <c r="G20" s="14" t="n"/>
       <c r="H20" s="14" t="n"/>
     </row>
@@ -1122,7 +1131,7 @@
       <c r="C21" s="6" t="n"/>
       <c r="D21" s="6" t="n"/>
       <c r="E21" s="6" t="n"/>
-      <c r="F21" s="16" t="n"/>
+      <c r="F21" s="18" t="n"/>
       <c r="G21" s="6" t="n"/>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -1132,7 +1141,7 @@
       <c r="C22" s="14" t="n"/>
       <c r="D22" s="14" t="n"/>
       <c r="E22" s="14" t="n"/>
-      <c r="F22" s="15" t="n"/>
+      <c r="F22" s="17" t="n"/>
       <c r="G22" s="14" t="n"/>
       <c r="H22" s="14" t="n"/>
     </row>
@@ -1142,7 +1151,7 @@
       <c r="C23" s="6" t="n"/>
       <c r="D23" s="6" t="n"/>
       <c r="E23" s="6" t="n"/>
-      <c r="F23" s="16" t="n"/>
+      <c r="F23" s="18" t="n"/>
       <c r="G23" s="6" t="n"/>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -1152,7 +1161,7 @@
       <c r="C24" s="14" t="n"/>
       <c r="D24" s="14" t="n"/>
       <c r="E24" s="14" t="n"/>
-      <c r="F24" s="15" t="n"/>
+      <c r="F24" s="17" t="n"/>
       <c r="G24" s="14" t="n"/>
       <c r="H24" s="14" t="n"/>
     </row>
@@ -1162,7 +1171,7 @@
       <c r="C25" s="6" t="n"/>
       <c r="D25" s="6" t="n"/>
       <c r="E25" s="6" t="n"/>
-      <c r="F25" s="16" t="n"/>
+      <c r="F25" s="18" t="n"/>
       <c r="G25" s="6" t="n"/>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -1172,7 +1181,7 @@
       <c r="C26" s="14" t="n"/>
       <c r="D26" s="14" t="n"/>
       <c r="E26" s="14" t="n"/>
-      <c r="F26" s="15" t="n"/>
+      <c r="F26" s="17" t="n"/>
       <c r="G26" s="14" t="n"/>
       <c r="H26" s="14" t="n"/>
     </row>
@@ -1182,7 +1191,7 @@
       <c r="C27" s="6" t="n"/>
       <c r="D27" s="6" t="n"/>
       <c r="E27" s="6" t="n"/>
-      <c r="F27" s="16" t="n"/>
+      <c r="F27" s="18" t="n"/>
       <c r="G27" s="6" t="n"/>
       <c r="H27" s="6" t="n"/>
     </row>
@@ -1192,7 +1201,7 @@
       <c r="C28" s="14" t="n"/>
       <c r="D28" s="14" t="n"/>
       <c r="E28" s="14" t="n"/>
-      <c r="F28" s="15" t="n"/>
+      <c r="F28" s="17" t="n"/>
       <c r="G28" s="14" t="n"/>
       <c r="H28" s="14" t="n"/>
     </row>
@@ -1202,7 +1211,7 @@
       <c r="C29" s="6" t="n"/>
       <c r="D29" s="6" t="n"/>
       <c r="E29" s="6" t="n"/>
-      <c r="F29" s="16" t="n"/>
+      <c r="F29" s="18" t="n"/>
       <c r="G29" s="6" t="n"/>
       <c r="H29" s="6" t="n"/>
     </row>
@@ -1212,7 +1221,7 @@
       <c r="C30" s="14" t="n"/>
       <c r="D30" s="14" t="n"/>
       <c r="E30" s="14" t="n"/>
-      <c r="F30" s="15" t="n"/>
+      <c r="F30" s="17" t="n"/>
       <c r="G30" s="14" t="n"/>
       <c r="H30" s="14" t="n"/>
     </row>
@@ -1222,7 +1231,7 @@
       <c r="C31" s="6" t="n"/>
       <c r="D31" s="6" t="n"/>
       <c r="E31" s="6" t="n"/>
-      <c r="F31" s="16" t="n"/>
+      <c r="F31" s="18" t="n"/>
       <c r="G31" s="6" t="n"/>
       <c r="H31" s="6" t="n"/>
     </row>
@@ -1232,7 +1241,7 @@
       <c r="C32" s="14" t="n"/>
       <c r="D32" s="14" t="n"/>
       <c r="E32" s="14" t="n"/>
-      <c r="F32" s="15" t="n"/>
+      <c r="F32" s="17" t="n"/>
       <c r="G32" s="14" t="n"/>
       <c r="H32" s="14" t="n"/>
     </row>
@@ -1242,7 +1251,7 @@
       <c r="C33" s="6" t="n"/>
       <c r="D33" s="6" t="n"/>
       <c r="E33" s="6" t="n"/>
-      <c r="F33" s="16" t="n"/>
+      <c r="F33" s="18" t="n"/>
       <c r="G33" s="6" t="n"/>
       <c r="H33" s="6" t="n"/>
     </row>
@@ -1252,7 +1261,7 @@
       <c r="C34" s="14" t="n"/>
       <c r="D34" s="14" t="n"/>
       <c r="E34" s="14" t="n"/>
-      <c r="F34" s="15" t="n"/>
+      <c r="F34" s="17" t="n"/>
       <c r="G34" s="14" t="n"/>
       <c r="H34" s="14" t="n"/>
     </row>
@@ -1262,7 +1271,7 @@
       <c r="C35" s="6" t="n"/>
       <c r="D35" s="6" t="n"/>
       <c r="E35" s="6" t="n"/>
-      <c r="F35" s="16" t="n"/>
+      <c r="F35" s="18" t="n"/>
       <c r="G35" s="6" t="n"/>
       <c r="H35" s="6" t="n"/>
     </row>
@@ -1272,7 +1281,7 @@
       <c r="C36" s="14" t="n"/>
       <c r="D36" s="14" t="n"/>
       <c r="E36" s="14" t="n"/>
-      <c r="F36" s="15" t="n"/>
+      <c r="F36" s="17" t="n"/>
       <c r="G36" s="14" t="n"/>
       <c r="H36" s="14" t="n"/>
     </row>
@@ -1282,7 +1291,7 @@
       <c r="C37" s="6" t="n"/>
       <c r="D37" s="6" t="n"/>
       <c r="E37" s="6" t="n"/>
-      <c r="F37" s="16" t="n"/>
+      <c r="F37" s="18" t="n"/>
       <c r="G37" s="6" t="n"/>
       <c r="H37" s="6" t="n"/>
     </row>
@@ -1292,7 +1301,7 @@
       <c r="C38" s="14" t="n"/>
       <c r="D38" s="14" t="n"/>
       <c r="E38" s="14" t="n"/>
-      <c r="F38" s="15" t="n"/>
+      <c r="F38" s="17" t="n"/>
       <c r="G38" s="14" t="n"/>
       <c r="H38" s="14" t="n"/>
     </row>
@@ -1302,7 +1311,7 @@
       <c r="C39" s="6" t="n"/>
       <c r="D39" s="6" t="n"/>
       <c r="E39" s="6" t="n"/>
-      <c r="F39" s="16" t="n"/>
+      <c r="F39" s="18" t="n"/>
       <c r="G39" s="6" t="n"/>
       <c r="H39" s="6" t="n"/>
     </row>
@@ -1312,7 +1321,7 @@
       <c r="C40" s="14" t="n"/>
       <c r="D40" s="14" t="n"/>
       <c r="E40" s="14" t="n"/>
-      <c r="F40" s="15" t="n"/>
+      <c r="F40" s="17" t="n"/>
       <c r="G40" s="14" t="n"/>
       <c r="H40" s="14" t="n"/>
     </row>
@@ -1322,7 +1331,7 @@
       <c r="C41" s="6" t="n"/>
       <c r="D41" s="6" t="n"/>
       <c r="E41" s="6" t="n"/>
-      <c r="F41" s="16" t="n"/>
+      <c r="F41" s="18" t="n"/>
       <c r="G41" s="6" t="n"/>
       <c r="H41" s="6" t="n"/>
     </row>
@@ -1332,7 +1341,7 @@
       <c r="C42" s="14" t="n"/>
       <c r="D42" s="14" t="n"/>
       <c r="E42" s="14" t="n"/>
-      <c r="F42" s="15" t="n"/>
+      <c r="F42" s="17" t="n"/>
       <c r="G42" s="14" t="n"/>
       <c r="H42" s="14" t="n"/>
     </row>
@@ -1342,7 +1351,7 @@
       <c r="C43" s="6" t="n"/>
       <c r="D43" s="6" t="n"/>
       <c r="E43" s="6" t="n"/>
-      <c r="F43" s="16" t="n"/>
+      <c r="F43" s="18" t="n"/>
       <c r="G43" s="6" t="n"/>
       <c r="H43" s="6" t="n"/>
     </row>
@@ -1452,10 +1461,10 @@
           <t>XYZ Franchisee</t>
         </is>
       </c>
-      <c r="E2" s="15" t="n">
+      <c r="E2" s="17" t="n">
         <v>46023</v>
       </c>
-      <c r="F2" s="15" t="n">
+      <c r="F2" s="17" t="n">
         <v>46388</v>
       </c>
       <c r="G2" s="14">
@@ -1493,10 +1502,10 @@
           <t>Property Owner</t>
         </is>
       </c>
-      <c r="E3" s="16" t="n">
+      <c r="E3" s="18" t="n">
         <v>45873</v>
       </c>
-      <c r="F3" s="16" t="n">
+      <c r="F3" s="18" t="n">
         <v>46238</v>
       </c>
       <c r="G3" s="6">
@@ -1520,8 +1529,8 @@
       <c r="B4" s="14" t="n"/>
       <c r="C4" s="14" t="n"/>
       <c r="D4" s="14" t="n"/>
-      <c r="E4" s="15" t="n"/>
-      <c r="F4" s="15" t="n"/>
+      <c r="E4" s="17" t="n"/>
+      <c r="F4" s="17" t="n"/>
       <c r="G4" s="14">
         <f>IF(F4="","",F4-TODAY())</f>
         <v/>
@@ -1535,8 +1544,8 @@
       <c r="B5" s="6" t="n"/>
       <c r="C5" s="6" t="n"/>
       <c r="D5" s="6" t="n"/>
-      <c r="E5" s="16" t="n"/>
-      <c r="F5" s="16" t="n"/>
+      <c r="E5" s="18" t="n"/>
+      <c r="F5" s="18" t="n"/>
       <c r="G5" s="6">
         <f>IF(F5="","",F5-TODAY())</f>
         <v/>
@@ -1550,8 +1559,8 @@
       <c r="B6" s="14" t="n"/>
       <c r="C6" s="14" t="n"/>
       <c r="D6" s="14" t="n"/>
-      <c r="E6" s="15" t="n"/>
-      <c r="F6" s="15" t="n"/>
+      <c r="E6" s="17" t="n"/>
+      <c r="F6" s="17" t="n"/>
       <c r="G6" s="14">
         <f>IF(F6="","",F6-TODAY())</f>
         <v/>
@@ -1565,8 +1574,8 @@
       <c r="B7" s="6" t="n"/>
       <c r="C7" s="6" t="n"/>
       <c r="D7" s="6" t="n"/>
-      <c r="E7" s="16" t="n"/>
-      <c r="F7" s="16" t="n"/>
+      <c r="E7" s="18" t="n"/>
+      <c r="F7" s="18" t="n"/>
       <c r="G7" s="6">
         <f>IF(F7="","",F7-TODAY())</f>
         <v/>
@@ -1580,8 +1589,8 @@
       <c r="B8" s="14" t="n"/>
       <c r="C8" s="14" t="n"/>
       <c r="D8" s="14" t="n"/>
-      <c r="E8" s="15" t="n"/>
-      <c r="F8" s="15" t="n"/>
+      <c r="E8" s="17" t="n"/>
+      <c r="F8" s="17" t="n"/>
       <c r="G8" s="14">
         <f>IF(F8="","",F8-TODAY())</f>
         <v/>
@@ -1595,8 +1604,8 @@
       <c r="B9" s="6" t="n"/>
       <c r="C9" s="6" t="n"/>
       <c r="D9" s="6" t="n"/>
-      <c r="E9" s="16" t="n"/>
-      <c r="F9" s="16" t="n"/>
+      <c r="E9" s="18" t="n"/>
+      <c r="F9" s="18" t="n"/>
       <c r="G9" s="6">
         <f>IF(F9="","",F9-TODAY())</f>
         <v/>
@@ -1610,8 +1619,8 @@
       <c r="B10" s="14" t="n"/>
       <c r="C10" s="14" t="n"/>
       <c r="D10" s="14" t="n"/>
-      <c r="E10" s="15" t="n"/>
-      <c r="F10" s="15" t="n"/>
+      <c r="E10" s="17" t="n"/>
+      <c r="F10" s="17" t="n"/>
       <c r="G10" s="14">
         <f>IF(F10="","",F10-TODAY())</f>
         <v/>
@@ -1625,8 +1634,8 @@
       <c r="B11" s="6" t="n"/>
       <c r="C11" s="6" t="n"/>
       <c r="D11" s="6" t="n"/>
-      <c r="E11" s="16" t="n"/>
-      <c r="F11" s="16" t="n"/>
+      <c r="E11" s="18" t="n"/>
+      <c r="F11" s="18" t="n"/>
       <c r="G11" s="6">
         <f>IF(F11="","",F11-TODAY())</f>
         <v/>
@@ -1640,8 +1649,8 @@
       <c r="B12" s="14" t="n"/>
       <c r="C12" s="14" t="n"/>
       <c r="D12" s="14" t="n"/>
-      <c r="E12" s="15" t="n"/>
-      <c r="F12" s="15" t="n"/>
+      <c r="E12" s="17" t="n"/>
+      <c r="F12" s="17" t="n"/>
       <c r="G12" s="14">
         <f>IF(F12="","",F12-TODAY())</f>
         <v/>
@@ -1655,8 +1664,8 @@
       <c r="B13" s="6" t="n"/>
       <c r="C13" s="6" t="n"/>
       <c r="D13" s="6" t="n"/>
-      <c r="E13" s="16" t="n"/>
-      <c r="F13" s="16" t="n"/>
+      <c r="E13" s="18" t="n"/>
+      <c r="F13" s="18" t="n"/>
       <c r="G13" s="6">
         <f>IF(F13="","",F13-TODAY())</f>
         <v/>
@@ -1670,8 +1679,8 @@
       <c r="B14" s="14" t="n"/>
       <c r="C14" s="14" t="n"/>
       <c r="D14" s="14" t="n"/>
-      <c r="E14" s="15" t="n"/>
-      <c r="F14" s="15" t="n"/>
+      <c r="E14" s="17" t="n"/>
+      <c r="F14" s="17" t="n"/>
       <c r="G14" s="14">
         <f>IF(F14="","",F14-TODAY())</f>
         <v/>
@@ -1685,8 +1694,8 @@
       <c r="B15" s="6" t="n"/>
       <c r="C15" s="6" t="n"/>
       <c r="D15" s="6" t="n"/>
-      <c r="E15" s="16" t="n"/>
-      <c r="F15" s="16" t="n"/>
+      <c r="E15" s="18" t="n"/>
+      <c r="F15" s="18" t="n"/>
       <c r="G15" s="6">
         <f>IF(F15="","",F15-TODAY())</f>
         <v/>
@@ -1700,8 +1709,8 @@
       <c r="B16" s="14" t="n"/>
       <c r="C16" s="14" t="n"/>
       <c r="D16" s="14" t="n"/>
-      <c r="E16" s="15" t="n"/>
-      <c r="F16" s="15" t="n"/>
+      <c r="E16" s="17" t="n"/>
+      <c r="F16" s="17" t="n"/>
       <c r="G16" s="14">
         <f>IF(F16="","",F16-TODAY())</f>
         <v/>
@@ -1715,8 +1724,8 @@
       <c r="B17" s="6" t="n"/>
       <c r="C17" s="6" t="n"/>
       <c r="D17" s="6" t="n"/>
-      <c r="E17" s="16" t="n"/>
-      <c r="F17" s="16" t="n"/>
+      <c r="E17" s="18" t="n"/>
+      <c r="F17" s="18" t="n"/>
       <c r="G17" s="6">
         <f>IF(F17="","",F17-TODAY())</f>
         <v/>
@@ -1730,8 +1739,8 @@
       <c r="B18" s="14" t="n"/>
       <c r="C18" s="14" t="n"/>
       <c r="D18" s="14" t="n"/>
-      <c r="E18" s="15" t="n"/>
-      <c r="F18" s="15" t="n"/>
+      <c r="E18" s="17" t="n"/>
+      <c r="F18" s="17" t="n"/>
       <c r="G18" s="14">
         <f>IF(F18="","",F18-TODAY())</f>
         <v/>
@@ -1745,8 +1754,8 @@
       <c r="B19" s="6" t="n"/>
       <c r="C19" s="6" t="n"/>
       <c r="D19" s="6" t="n"/>
-      <c r="E19" s="16" t="n"/>
-      <c r="F19" s="16" t="n"/>
+      <c r="E19" s="18" t="n"/>
+      <c r="F19" s="18" t="n"/>
       <c r="G19" s="6">
         <f>IF(F19="","",F19-TODAY())</f>
         <v/>
@@ -1760,8 +1769,8 @@
       <c r="B20" s="14" t="n"/>
       <c r="C20" s="14" t="n"/>
       <c r="D20" s="14" t="n"/>
-      <c r="E20" s="15" t="n"/>
-      <c r="F20" s="15" t="n"/>
+      <c r="E20" s="17" t="n"/>
+      <c r="F20" s="17" t="n"/>
       <c r="G20" s="14">
         <f>IF(F20="","",F20-TODAY())</f>
         <v/>
@@ -1775,8 +1784,8 @@
       <c r="B21" s="6" t="n"/>
       <c r="C21" s="6" t="n"/>
       <c r="D21" s="6" t="n"/>
-      <c r="E21" s="16" t="n"/>
-      <c r="F21" s="16" t="n"/>
+      <c r="E21" s="18" t="n"/>
+      <c r="F21" s="18" t="n"/>
       <c r="G21" s="6">
         <f>IF(F21="","",F21-TODAY())</f>
         <v/>
@@ -1790,8 +1799,8 @@
       <c r="B22" s="14" t="n"/>
       <c r="C22" s="14" t="n"/>
       <c r="D22" s="14" t="n"/>
-      <c r="E22" s="15" t="n"/>
-      <c r="F22" s="15" t="n"/>
+      <c r="E22" s="17" t="n"/>
+      <c r="F22" s="17" t="n"/>
       <c r="G22" s="14">
         <f>IF(F22="","",F22-TODAY())</f>
         <v/>
@@ -1805,8 +1814,8 @@
       <c r="B23" s="6" t="n"/>
       <c r="C23" s="6" t="n"/>
       <c r="D23" s="6" t="n"/>
-      <c r="E23" s="16" t="n"/>
-      <c r="F23" s="16" t="n"/>
+      <c r="E23" s="18" t="n"/>
+      <c r="F23" s="18" t="n"/>
       <c r="G23" s="6">
         <f>IF(F23="","",F23-TODAY())</f>
         <v/>
@@ -1820,8 +1829,8 @@
       <c r="B24" s="14" t="n"/>
       <c r="C24" s="14" t="n"/>
       <c r="D24" s="14" t="n"/>
-      <c r="E24" s="15" t="n"/>
-      <c r="F24" s="15" t="n"/>
+      <c r="E24" s="17" t="n"/>
+      <c r="F24" s="17" t="n"/>
       <c r="G24" s="14">
         <f>IF(F24="","",F24-TODAY())</f>
         <v/>
@@ -1835,8 +1844,8 @@
       <c r="B25" s="6" t="n"/>
       <c r="C25" s="6" t="n"/>
       <c r="D25" s="6" t="n"/>
-      <c r="E25" s="16" t="n"/>
-      <c r="F25" s="16" t="n"/>
+      <c r="E25" s="18" t="n"/>
+      <c r="F25" s="18" t="n"/>
       <c r="G25" s="6">
         <f>IF(F25="","",F25-TODAY())</f>
         <v/>
@@ -1850,8 +1859,8 @@
       <c r="B26" s="14" t="n"/>
       <c r="C26" s="14" t="n"/>
       <c r="D26" s="14" t="n"/>
-      <c r="E26" s="15" t="n"/>
-      <c r="F26" s="15" t="n"/>
+      <c r="E26" s="17" t="n"/>
+      <c r="F26" s="17" t="n"/>
       <c r="G26" s="14">
         <f>IF(F26="","",F26-TODAY())</f>
         <v/>
@@ -1865,8 +1874,8 @@
       <c r="B27" s="6" t="n"/>
       <c r="C27" s="6" t="n"/>
       <c r="D27" s="6" t="n"/>
-      <c r="E27" s="16" t="n"/>
-      <c r="F27" s="16" t="n"/>
+      <c r="E27" s="18" t="n"/>
+      <c r="F27" s="18" t="n"/>
       <c r="G27" s="6">
         <f>IF(F27="","",F27-TODAY())</f>
         <v/>
@@ -1880,8 +1889,8 @@
       <c r="B28" s="14" t="n"/>
       <c r="C28" s="14" t="n"/>
       <c r="D28" s="14" t="n"/>
-      <c r="E28" s="15" t="n"/>
-      <c r="F28" s="15" t="n"/>
+      <c r="E28" s="17" t="n"/>
+      <c r="F28" s="17" t="n"/>
       <c r="G28" s="14">
         <f>IF(F28="","",F28-TODAY())</f>
         <v/>
@@ -1895,8 +1904,8 @@
       <c r="B29" s="6" t="n"/>
       <c r="C29" s="6" t="n"/>
       <c r="D29" s="6" t="n"/>
-      <c r="E29" s="16" t="n"/>
-      <c r="F29" s="16" t="n"/>
+      <c r="E29" s="18" t="n"/>
+      <c r="F29" s="18" t="n"/>
       <c r="G29" s="6">
         <f>IF(F29="","",F29-TODAY())</f>
         <v/>
@@ -1910,8 +1919,8 @@
       <c r="B30" s="14" t="n"/>
       <c r="C30" s="14" t="n"/>
       <c r="D30" s="14" t="n"/>
-      <c r="E30" s="15" t="n"/>
-      <c r="F30" s="15" t="n"/>
+      <c r="E30" s="17" t="n"/>
+      <c r="F30" s="17" t="n"/>
       <c r="G30" s="14">
         <f>IF(F30="","",F30-TODAY())</f>
         <v/>
@@ -1925,8 +1934,8 @@
       <c r="B31" s="6" t="n"/>
       <c r="C31" s="6" t="n"/>
       <c r="D31" s="6" t="n"/>
-      <c r="E31" s="16" t="n"/>
-      <c r="F31" s="16" t="n"/>
+      <c r="E31" s="18" t="n"/>
+      <c r="F31" s="18" t="n"/>
       <c r="G31" s="6">
         <f>IF(F31="","",F31-TODAY())</f>
         <v/>
@@ -1940,8 +1949,8 @@
       <c r="B32" s="14" t="n"/>
       <c r="C32" s="14" t="n"/>
       <c r="D32" s="14" t="n"/>
-      <c r="E32" s="15" t="n"/>
-      <c r="F32" s="15" t="n"/>
+      <c r="E32" s="17" t="n"/>
+      <c r="F32" s="17" t="n"/>
       <c r="G32" s="14">
         <f>IF(F32="","",F32-TODAY())</f>
         <v/>
@@ -1955,8 +1964,8 @@
       <c r="B33" s="6" t="n"/>
       <c r="C33" s="6" t="n"/>
       <c r="D33" s="6" t="n"/>
-      <c r="E33" s="16" t="n"/>
-      <c r="F33" s="16" t="n"/>
+      <c r="E33" s="18" t="n"/>
+      <c r="F33" s="18" t="n"/>
       <c r="G33" s="6">
         <f>IF(F33="","",F33-TODAY())</f>
         <v/>
@@ -1970,8 +1979,8 @@
       <c r="B34" s="14" t="n"/>
       <c r="C34" s="14" t="n"/>
       <c r="D34" s="14" t="n"/>
-      <c r="E34" s="15" t="n"/>
-      <c r="F34" s="15" t="n"/>
+      <c r="E34" s="17" t="n"/>
+      <c r="F34" s="17" t="n"/>
       <c r="G34" s="14">
         <f>IF(F34="","",F34-TODAY())</f>
         <v/>
@@ -1985,8 +1994,8 @@
       <c r="B35" s="6" t="n"/>
       <c r="C35" s="6" t="n"/>
       <c r="D35" s="6" t="n"/>
-      <c r="E35" s="16" t="n"/>
-      <c r="F35" s="16" t="n"/>
+      <c r="E35" s="18" t="n"/>
+      <c r="F35" s="18" t="n"/>
       <c r="G35" s="6">
         <f>IF(F35="","",F35-TODAY())</f>
         <v/>
@@ -2000,8 +2009,8 @@
       <c r="B36" s="14" t="n"/>
       <c r="C36" s="14" t="n"/>
       <c r="D36" s="14" t="n"/>
-      <c r="E36" s="15" t="n"/>
-      <c r="F36" s="15" t="n"/>
+      <c r="E36" s="17" t="n"/>
+      <c r="F36" s="17" t="n"/>
       <c r="G36" s="14">
         <f>IF(F36="","",F36-TODAY())</f>
         <v/>
@@ -2015,8 +2024,8 @@
       <c r="B37" s="6" t="n"/>
       <c r="C37" s="6" t="n"/>
       <c r="D37" s="6" t="n"/>
-      <c r="E37" s="16" t="n"/>
-      <c r="F37" s="16" t="n"/>
+      <c r="E37" s="18" t="n"/>
+      <c r="F37" s="18" t="n"/>
       <c r="G37" s="6">
         <f>IF(F37="","",F37-TODAY())</f>
         <v/>
@@ -2030,8 +2039,8 @@
       <c r="B38" s="14" t="n"/>
       <c r="C38" s="14" t="n"/>
       <c r="D38" s="14" t="n"/>
-      <c r="E38" s="15" t="n"/>
-      <c r="F38" s="15" t="n"/>
+      <c r="E38" s="17" t="n"/>
+      <c r="F38" s="17" t="n"/>
       <c r="G38" s="14">
         <f>IF(F38="","",F38-TODAY())</f>
         <v/>
@@ -2045,8 +2054,8 @@
       <c r="B39" s="6" t="n"/>
       <c r="C39" s="6" t="n"/>
       <c r="D39" s="6" t="n"/>
-      <c r="E39" s="16" t="n"/>
-      <c r="F39" s="16" t="n"/>
+      <c r="E39" s="18" t="n"/>
+      <c r="F39" s="18" t="n"/>
       <c r="G39" s="6">
         <f>IF(F39="","",F39-TODAY())</f>
         <v/>
@@ -2060,8 +2069,8 @@
       <c r="B40" s="14" t="n"/>
       <c r="C40" s="14" t="n"/>
       <c r="D40" s="14" t="n"/>
-      <c r="E40" s="15" t="n"/>
-      <c r="F40" s="15" t="n"/>
+      <c r="E40" s="17" t="n"/>
+      <c r="F40" s="17" t="n"/>
       <c r="G40" s="14">
         <f>IF(F40="","",F40-TODAY())</f>
         <v/>
@@ -2075,8 +2084,8 @@
       <c r="B41" s="6" t="n"/>
       <c r="C41" s="6" t="n"/>
       <c r="D41" s="6" t="n"/>
-      <c r="E41" s="16" t="n"/>
-      <c r="F41" s="16" t="n"/>
+      <c r="E41" s="18" t="n"/>
+      <c r="F41" s="18" t="n"/>
       <c r="G41" s="6">
         <f>IF(F41="","",F41-TODAY())</f>
         <v/>
@@ -2090,8 +2099,8 @@
       <c r="B42" s="14" t="n"/>
       <c r="C42" s="14" t="n"/>
       <c r="D42" s="14" t="n"/>
-      <c r="E42" s="15" t="n"/>
-      <c r="F42" s="15" t="n"/>
+      <c r="E42" s="17" t="n"/>
+      <c r="F42" s="17" t="n"/>
       <c r="G42" s="14">
         <f>IF(F42="","",F42-TODAY())</f>
         <v/>
@@ -2105,8 +2114,8 @@
       <c r="B43" s="6" t="n"/>
       <c r="C43" s="6" t="n"/>
       <c r="D43" s="6" t="n"/>
-      <c r="E43" s="16" t="n"/>
-      <c r="F43" s="16" t="n"/>
+      <c r="E43" s="18" t="n"/>
+      <c r="F43" s="18" t="n"/>
       <c r="G43" s="6">
         <f>IF(F43="","",F43-TODAY())</f>
         <v/>
@@ -2213,24 +2222,24 @@
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>Sample Brand A</t>
+          <t>JS Concepts &amp; Solutions Pvt Ltd</t>
         </is>
       </c>
       <c r="C2" s="14" t="inlineStr">
         <is>
-          <t>12345678901234</t>
+          <t>22726442000324</t>
         </is>
       </c>
       <c r="D2" s="14" t="inlineStr">
         <is>
-          <t>State</t>
-        </is>
-      </c>
-      <c r="E2" s="15" t="n">
-        <v>45923</v>
-      </c>
-      <c r="F2" s="15" t="n">
-        <v>46288</v>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="E2" s="17" t="n">
+        <v>46151</v>
+      </c>
+      <c r="F2" s="17" t="n">
+        <v>46515</v>
       </c>
       <c r="G2" s="14">
         <f>IF(F2="","",F2-TODAY())</f>
@@ -2241,7 +2250,11 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="I2" s="14" t="inlineStr"/>
+      <c r="I2" s="14" t="inlineStr">
+        <is>
+          <t>Bennett University, TechZone II, Greater Noida. KOB: Petty Retailer snacks/tea. Tatkal reg. Renew annual fee before expiry.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="n">
@@ -2249,12 +2262,12 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>Outlet - MG Road</t>
+          <t>Parma Food &amp; Beverage (Jatin Jhawar)</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>10987654321098</t>
+          <t>22726442000472</t>
         </is>
       </c>
       <c r="D3" s="6" t="inlineStr">
@@ -2262,11 +2275,11 @@
           <t>Basic</t>
         </is>
       </c>
-      <c r="E3" s="16" t="n">
-        <v>45523</v>
-      </c>
-      <c r="F3" s="16" t="n">
+      <c r="E3" s="18" t="n">
         <v>46218</v>
+      </c>
+      <c r="F3" s="18" t="n">
+        <v>46582</v>
       </c>
       <c r="G3" s="6">
         <f>IF(F3="","",F3-TODAY())</f>
@@ -2274,12 +2287,12 @@
       </c>
       <c r="H3" s="6" t="inlineStr">
         <is>
-          <t>Expired</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="I3" s="6" t="inlineStr">
         <is>
-          <t>Renew immediately</t>
+          <t>Bennett University, TechZone 2, Greater Noida. KOB: Food Vending Agencies. Tatkal reg. Renew annual fee before expiry.</t>
         </is>
       </c>
     </row>
@@ -2288,8 +2301,8 @@
       <c r="B4" s="14" t="n"/>
       <c r="C4" s="14" t="n"/>
       <c r="D4" s="14" t="n"/>
-      <c r="E4" s="15" t="n"/>
-      <c r="F4" s="15" t="n"/>
+      <c r="E4" s="17" t="n"/>
+      <c r="F4" s="17" t="n"/>
       <c r="G4" s="14">
         <f>IF(F4="","",F4-TODAY())</f>
         <v/>
@@ -2302,8 +2315,8 @@
       <c r="B5" s="6" t="n"/>
       <c r="C5" s="6" t="n"/>
       <c r="D5" s="6" t="n"/>
-      <c r="E5" s="16" t="n"/>
-      <c r="F5" s="16" t="n"/>
+      <c r="E5" s="18" t="n"/>
+      <c r="F5" s="18" t="n"/>
       <c r="G5" s="6">
         <f>IF(F5="","",F5-TODAY())</f>
         <v/>
@@ -2316,8 +2329,8 @@
       <c r="B6" s="14" t="n"/>
       <c r="C6" s="14" t="n"/>
       <c r="D6" s="14" t="n"/>
-      <c r="E6" s="15" t="n"/>
-      <c r="F6" s="15" t="n"/>
+      <c r="E6" s="17" t="n"/>
+      <c r="F6" s="17" t="n"/>
       <c r="G6" s="14">
         <f>IF(F6="","",F6-TODAY())</f>
         <v/>
@@ -2330,8 +2343,8 @@
       <c r="B7" s="6" t="n"/>
       <c r="C7" s="6" t="n"/>
       <c r="D7" s="6" t="n"/>
-      <c r="E7" s="16" t="n"/>
-      <c r="F7" s="16" t="n"/>
+      <c r="E7" s="18" t="n"/>
+      <c r="F7" s="18" t="n"/>
       <c r="G7" s="6">
         <f>IF(F7="","",F7-TODAY())</f>
         <v/>
@@ -2344,8 +2357,8 @@
       <c r="B8" s="14" t="n"/>
       <c r="C8" s="14" t="n"/>
       <c r="D8" s="14" t="n"/>
-      <c r="E8" s="15" t="n"/>
-      <c r="F8" s="15" t="n"/>
+      <c r="E8" s="17" t="n"/>
+      <c r="F8" s="17" t="n"/>
       <c r="G8" s="14">
         <f>IF(F8="","",F8-TODAY())</f>
         <v/>
@@ -2358,8 +2371,8 @@
       <c r="B9" s="6" t="n"/>
       <c r="C9" s="6" t="n"/>
       <c r="D9" s="6" t="n"/>
-      <c r="E9" s="16" t="n"/>
-      <c r="F9" s="16" t="n"/>
+      <c r="E9" s="18" t="n"/>
+      <c r="F9" s="18" t="n"/>
       <c r="G9" s="6">
         <f>IF(F9="","",F9-TODAY())</f>
         <v/>
@@ -2372,8 +2385,8 @@
       <c r="B10" s="14" t="n"/>
       <c r="C10" s="14" t="n"/>
       <c r="D10" s="14" t="n"/>
-      <c r="E10" s="15" t="n"/>
-      <c r="F10" s="15" t="n"/>
+      <c r="E10" s="17" t="n"/>
+      <c r="F10" s="17" t="n"/>
       <c r="G10" s="14">
         <f>IF(F10="","",F10-TODAY())</f>
         <v/>
@@ -2386,8 +2399,8 @@
       <c r="B11" s="6" t="n"/>
       <c r="C11" s="6" t="n"/>
       <c r="D11" s="6" t="n"/>
-      <c r="E11" s="16" t="n"/>
-      <c r="F11" s="16" t="n"/>
+      <c r="E11" s="18" t="n"/>
+      <c r="F11" s="18" t="n"/>
       <c r="G11" s="6">
         <f>IF(F11="","",F11-TODAY())</f>
         <v/>
@@ -2400,8 +2413,8 @@
       <c r="B12" s="14" t="n"/>
       <c r="C12" s="14" t="n"/>
       <c r="D12" s="14" t="n"/>
-      <c r="E12" s="15" t="n"/>
-      <c r="F12" s="15" t="n"/>
+      <c r="E12" s="17" t="n"/>
+      <c r="F12" s="17" t="n"/>
       <c r="G12" s="14">
         <f>IF(F12="","",F12-TODAY())</f>
         <v/>
@@ -2414,8 +2427,8 @@
       <c r="B13" s="6" t="n"/>
       <c r="C13" s="6" t="n"/>
       <c r="D13" s="6" t="n"/>
-      <c r="E13" s="16" t="n"/>
-      <c r="F13" s="16" t="n"/>
+      <c r="E13" s="18" t="n"/>
+      <c r="F13" s="18" t="n"/>
       <c r="G13" s="6">
         <f>IF(F13="","",F13-TODAY())</f>
         <v/>
@@ -2428,8 +2441,8 @@
       <c r="B14" s="14" t="n"/>
       <c r="C14" s="14" t="n"/>
       <c r="D14" s="14" t="n"/>
-      <c r="E14" s="15" t="n"/>
-      <c r="F14" s="15" t="n"/>
+      <c r="E14" s="17" t="n"/>
+      <c r="F14" s="17" t="n"/>
       <c r="G14" s="14">
         <f>IF(F14="","",F14-TODAY())</f>
         <v/>
@@ -2442,8 +2455,8 @@
       <c r="B15" s="6" t="n"/>
       <c r="C15" s="6" t="n"/>
       <c r="D15" s="6" t="n"/>
-      <c r="E15" s="16" t="n"/>
-      <c r="F15" s="16" t="n"/>
+      <c r="E15" s="18" t="n"/>
+      <c r="F15" s="18" t="n"/>
       <c r="G15" s="6">
         <f>IF(F15="","",F15-TODAY())</f>
         <v/>
@@ -2456,8 +2469,8 @@
       <c r="B16" s="14" t="n"/>
       <c r="C16" s="14" t="n"/>
       <c r="D16" s="14" t="n"/>
-      <c r="E16" s="15" t="n"/>
-      <c r="F16" s="15" t="n"/>
+      <c r="E16" s="17" t="n"/>
+      <c r="F16" s="17" t="n"/>
       <c r="G16" s="14">
         <f>IF(F16="","",F16-TODAY())</f>
         <v/>
@@ -2470,8 +2483,8 @@
       <c r="B17" s="6" t="n"/>
       <c r="C17" s="6" t="n"/>
       <c r="D17" s="6" t="n"/>
-      <c r="E17" s="16" t="n"/>
-      <c r="F17" s="16" t="n"/>
+      <c r="E17" s="18" t="n"/>
+      <c r="F17" s="18" t="n"/>
       <c r="G17" s="6">
         <f>IF(F17="","",F17-TODAY())</f>
         <v/>
@@ -2484,8 +2497,8 @@
       <c r="B18" s="14" t="n"/>
       <c r="C18" s="14" t="n"/>
       <c r="D18" s="14" t="n"/>
-      <c r="E18" s="15" t="n"/>
-      <c r="F18" s="15" t="n"/>
+      <c r="E18" s="17" t="n"/>
+      <c r="F18" s="17" t="n"/>
       <c r="G18" s="14">
         <f>IF(F18="","",F18-TODAY())</f>
         <v/>
@@ -2498,8 +2511,8 @@
       <c r="B19" s="6" t="n"/>
       <c r="C19" s="6" t="n"/>
       <c r="D19" s="6" t="n"/>
-      <c r="E19" s="16" t="n"/>
-      <c r="F19" s="16" t="n"/>
+      <c r="E19" s="18" t="n"/>
+      <c r="F19" s="18" t="n"/>
       <c r="G19" s="6">
         <f>IF(F19="","",F19-TODAY())</f>
         <v/>
@@ -2512,8 +2525,8 @@
       <c r="B20" s="14" t="n"/>
       <c r="C20" s="14" t="n"/>
       <c r="D20" s="14" t="n"/>
-      <c r="E20" s="15" t="n"/>
-      <c r="F20" s="15" t="n"/>
+      <c r="E20" s="17" t="n"/>
+      <c r="F20" s="17" t="n"/>
       <c r="G20" s="14">
         <f>IF(F20="","",F20-TODAY())</f>
         <v/>
@@ -2526,8 +2539,8 @@
       <c r="B21" s="6" t="n"/>
       <c r="C21" s="6" t="n"/>
       <c r="D21" s="6" t="n"/>
-      <c r="E21" s="16" t="n"/>
-      <c r="F21" s="16" t="n"/>
+      <c r="E21" s="18" t="n"/>
+      <c r="F21" s="18" t="n"/>
       <c r="G21" s="6">
         <f>IF(F21="","",F21-TODAY())</f>
         <v/>
@@ -2540,8 +2553,8 @@
       <c r="B22" s="14" t="n"/>
       <c r="C22" s="14" t="n"/>
       <c r="D22" s="14" t="n"/>
-      <c r="E22" s="15" t="n"/>
-      <c r="F22" s="15" t="n"/>
+      <c r="E22" s="17" t="n"/>
+      <c r="F22" s="17" t="n"/>
       <c r="G22" s="14">
         <f>IF(F22="","",F22-TODAY())</f>
         <v/>
@@ -2554,8 +2567,8 @@
       <c r="B23" s="6" t="n"/>
       <c r="C23" s="6" t="n"/>
       <c r="D23" s="6" t="n"/>
-      <c r="E23" s="16" t="n"/>
-      <c r="F23" s="16" t="n"/>
+      <c r="E23" s="18" t="n"/>
+      <c r="F23" s="18" t="n"/>
       <c r="G23" s="6">
         <f>IF(F23="","",F23-TODAY())</f>
         <v/>
@@ -2568,8 +2581,8 @@
       <c r="B24" s="14" t="n"/>
       <c r="C24" s="14" t="n"/>
       <c r="D24" s="14" t="n"/>
-      <c r="E24" s="15" t="n"/>
-      <c r="F24" s="15" t="n"/>
+      <c r="E24" s="17" t="n"/>
+      <c r="F24" s="17" t="n"/>
       <c r="G24" s="14">
         <f>IF(F24="","",F24-TODAY())</f>
         <v/>
@@ -2582,8 +2595,8 @@
       <c r="B25" s="6" t="n"/>
       <c r="C25" s="6" t="n"/>
       <c r="D25" s="6" t="n"/>
-      <c r="E25" s="16" t="n"/>
-      <c r="F25" s="16" t="n"/>
+      <c r="E25" s="18" t="n"/>
+      <c r="F25" s="18" t="n"/>
       <c r="G25" s="6">
         <f>IF(F25="","",F25-TODAY())</f>
         <v/>
@@ -2596,8 +2609,8 @@
       <c r="B26" s="14" t="n"/>
       <c r="C26" s="14" t="n"/>
       <c r="D26" s="14" t="n"/>
-      <c r="E26" s="15" t="n"/>
-      <c r="F26" s="15" t="n"/>
+      <c r="E26" s="17" t="n"/>
+      <c r="F26" s="17" t="n"/>
       <c r="G26" s="14">
         <f>IF(F26="","",F26-TODAY())</f>
         <v/>
@@ -2610,8 +2623,8 @@
       <c r="B27" s="6" t="n"/>
       <c r="C27" s="6" t="n"/>
       <c r="D27" s="6" t="n"/>
-      <c r="E27" s="16" t="n"/>
-      <c r="F27" s="16" t="n"/>
+      <c r="E27" s="18" t="n"/>
+      <c r="F27" s="18" t="n"/>
       <c r="G27" s="6">
         <f>IF(F27="","",F27-TODAY())</f>
         <v/>
@@ -2624,8 +2637,8 @@
       <c r="B28" s="14" t="n"/>
       <c r="C28" s="14" t="n"/>
       <c r="D28" s="14" t="n"/>
-      <c r="E28" s="15" t="n"/>
-      <c r="F28" s="15" t="n"/>
+      <c r="E28" s="17" t="n"/>
+      <c r="F28" s="17" t="n"/>
       <c r="G28" s="14">
         <f>IF(F28="","",F28-TODAY())</f>
         <v/>
@@ -2638,8 +2651,8 @@
       <c r="B29" s="6" t="n"/>
       <c r="C29" s="6" t="n"/>
       <c r="D29" s="6" t="n"/>
-      <c r="E29" s="16" t="n"/>
-      <c r="F29" s="16" t="n"/>
+      <c r="E29" s="18" t="n"/>
+      <c r="F29" s="18" t="n"/>
       <c r="G29" s="6">
         <f>IF(F29="","",F29-TODAY())</f>
         <v/>
@@ -2652,8 +2665,8 @@
       <c r="B30" s="14" t="n"/>
       <c r="C30" s="14" t="n"/>
       <c r="D30" s="14" t="n"/>
-      <c r="E30" s="15" t="n"/>
-      <c r="F30" s="15" t="n"/>
+      <c r="E30" s="17" t="n"/>
+      <c r="F30" s="17" t="n"/>
       <c r="G30" s="14">
         <f>IF(F30="","",F30-TODAY())</f>
         <v/>
@@ -2666,8 +2679,8 @@
       <c r="B31" s="6" t="n"/>
       <c r="C31" s="6" t="n"/>
       <c r="D31" s="6" t="n"/>
-      <c r="E31" s="16" t="n"/>
-      <c r="F31" s="16" t="n"/>
+      <c r="E31" s="18" t="n"/>
+      <c r="F31" s="18" t="n"/>
       <c r="G31" s="6">
         <f>IF(F31="","",F31-TODAY())</f>
         <v/>
@@ -2680,8 +2693,8 @@
       <c r="B32" s="14" t="n"/>
       <c r="C32" s="14" t="n"/>
       <c r="D32" s="14" t="n"/>
-      <c r="E32" s="15" t="n"/>
-      <c r="F32" s="15" t="n"/>
+      <c r="E32" s="17" t="n"/>
+      <c r="F32" s="17" t="n"/>
       <c r="G32" s="14">
         <f>IF(F32="","",F32-TODAY())</f>
         <v/>
@@ -2694,8 +2707,8 @@
       <c r="B33" s="6" t="n"/>
       <c r="C33" s="6" t="n"/>
       <c r="D33" s="6" t="n"/>
-      <c r="E33" s="16" t="n"/>
-      <c r="F33" s="16" t="n"/>
+      <c r="E33" s="18" t="n"/>
+      <c r="F33" s="18" t="n"/>
       <c r="G33" s="6">
         <f>IF(F33="","",F33-TODAY())</f>
         <v/>
@@ -2708,8 +2721,8 @@
       <c r="B34" s="14" t="n"/>
       <c r="C34" s="14" t="n"/>
       <c r="D34" s="14" t="n"/>
-      <c r="E34" s="15" t="n"/>
-      <c r="F34" s="15" t="n"/>
+      <c r="E34" s="17" t="n"/>
+      <c r="F34" s="17" t="n"/>
       <c r="G34" s="14">
         <f>IF(F34="","",F34-TODAY())</f>
         <v/>
@@ -2722,8 +2735,8 @@
       <c r="B35" s="6" t="n"/>
       <c r="C35" s="6" t="n"/>
       <c r="D35" s="6" t="n"/>
-      <c r="E35" s="16" t="n"/>
-      <c r="F35" s="16" t="n"/>
+      <c r="E35" s="18" t="n"/>
+      <c r="F35" s="18" t="n"/>
       <c r="G35" s="6">
         <f>IF(F35="","",F35-TODAY())</f>
         <v/>
@@ -2736,8 +2749,8 @@
       <c r="B36" s="14" t="n"/>
       <c r="C36" s="14" t="n"/>
       <c r="D36" s="14" t="n"/>
-      <c r="E36" s="15" t="n"/>
-      <c r="F36" s="15" t="n"/>
+      <c r="E36" s="17" t="n"/>
+      <c r="F36" s="17" t="n"/>
       <c r="G36" s="14">
         <f>IF(F36="","",F36-TODAY())</f>
         <v/>
@@ -2750,8 +2763,8 @@
       <c r="B37" s="6" t="n"/>
       <c r="C37" s="6" t="n"/>
       <c r="D37" s="6" t="n"/>
-      <c r="E37" s="16" t="n"/>
-      <c r="F37" s="16" t="n"/>
+      <c r="E37" s="18" t="n"/>
+      <c r="F37" s="18" t="n"/>
       <c r="G37" s="6">
         <f>IF(F37="","",F37-TODAY())</f>
         <v/>
@@ -2764,8 +2777,8 @@
       <c r="B38" s="14" t="n"/>
       <c r="C38" s="14" t="n"/>
       <c r="D38" s="14" t="n"/>
-      <c r="E38" s="15" t="n"/>
-      <c r="F38" s="15" t="n"/>
+      <c r="E38" s="17" t="n"/>
+      <c r="F38" s="17" t="n"/>
       <c r="G38" s="14">
         <f>IF(F38="","",F38-TODAY())</f>
         <v/>
@@ -2778,8 +2791,8 @@
       <c r="B39" s="6" t="n"/>
       <c r="C39" s="6" t="n"/>
       <c r="D39" s="6" t="n"/>
-      <c r="E39" s="16" t="n"/>
-      <c r="F39" s="16" t="n"/>
+      <c r="E39" s="18" t="n"/>
+      <c r="F39" s="18" t="n"/>
       <c r="G39" s="6">
         <f>IF(F39="","",F39-TODAY())</f>
         <v/>
@@ -2792,8 +2805,8 @@
       <c r="B40" s="14" t="n"/>
       <c r="C40" s="14" t="n"/>
       <c r="D40" s="14" t="n"/>
-      <c r="E40" s="15" t="n"/>
-      <c r="F40" s="15" t="n"/>
+      <c r="E40" s="17" t="n"/>
+      <c r="F40" s="17" t="n"/>
       <c r="G40" s="14">
         <f>IF(F40="","",F40-TODAY())</f>
         <v/>
@@ -2806,8 +2819,8 @@
       <c r="B41" s="6" t="n"/>
       <c r="C41" s="6" t="n"/>
       <c r="D41" s="6" t="n"/>
-      <c r="E41" s="16" t="n"/>
-      <c r="F41" s="16" t="n"/>
+      <c r="E41" s="18" t="n"/>
+      <c r="F41" s="18" t="n"/>
       <c r="G41" s="6">
         <f>IF(F41="","",F41-TODAY())</f>
         <v/>
@@ -2820,8 +2833,8 @@
       <c r="B42" s="14" t="n"/>
       <c r="C42" s="14" t="n"/>
       <c r="D42" s="14" t="n"/>
-      <c r="E42" s="15" t="n"/>
-      <c r="F42" s="15" t="n"/>
+      <c r="E42" s="17" t="n"/>
+      <c r="F42" s="17" t="n"/>
       <c r="G42" s="14">
         <f>IF(F42="","",F42-TODAY())</f>
         <v/>
@@ -2834,8 +2847,8 @@
       <c r="B43" s="6" t="n"/>
       <c r="C43" s="6" t="n"/>
       <c r="D43" s="6" t="n"/>
-      <c r="E43" s="16" t="n"/>
-      <c r="F43" s="16" t="n"/>
+      <c r="E43" s="18" t="n"/>
+      <c r="F43" s="18" t="n"/>
       <c r="G43" s="6">
         <f>IF(F43="","",F43-TODAY())</f>
         <v/>
@@ -2977,7 +2990,7 @@
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="H2" s="15" t="n">
+      <c r="H2" s="17" t="n">
         <v>46043</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
@@ -3023,7 +3036,7 @@
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="H3" s="16" t="n">
+      <c r="H3" s="18" t="n">
         <v>46133</v>
       </c>
       <c r="I3" s="6" t="inlineStr">
@@ -3041,7 +3054,7 @@
       <c r="E4" s="14" t="n"/>
       <c r="F4" s="14" t="n"/>
       <c r="G4" s="14" t="n"/>
-      <c r="H4" s="15" t="n"/>
+      <c r="H4" s="17" t="n"/>
       <c r="I4" s="14" t="n"/>
       <c r="J4" s="14" t="n"/>
     </row>
@@ -3053,7 +3066,7 @@
       <c r="E5" s="6" t="n"/>
       <c r="F5" s="6" t="n"/>
       <c r="G5" s="6" t="n"/>
-      <c r="H5" s="16" t="n"/>
+      <c r="H5" s="18" t="n"/>
       <c r="I5" s="6" t="n"/>
       <c r="J5" s="6" t="n"/>
     </row>
@@ -3065,7 +3078,7 @@
       <c r="E6" s="14" t="n"/>
       <c r="F6" s="14" t="n"/>
       <c r="G6" s="14" t="n"/>
-      <c r="H6" s="15" t="n"/>
+      <c r="H6" s="17" t="n"/>
       <c r="I6" s="14" t="n"/>
       <c r="J6" s="14" t="n"/>
     </row>
@@ -3077,7 +3090,7 @@
       <c r="E7" s="6" t="n"/>
       <c r="F7" s="6" t="n"/>
       <c r="G7" s="6" t="n"/>
-      <c r="H7" s="16" t="n"/>
+      <c r="H7" s="18" t="n"/>
       <c r="I7" s="6" t="n"/>
       <c r="J7" s="6" t="n"/>
     </row>
@@ -3089,7 +3102,7 @@
       <c r="E8" s="14" t="n"/>
       <c r="F8" s="14" t="n"/>
       <c r="G8" s="14" t="n"/>
-      <c r="H8" s="15" t="n"/>
+      <c r="H8" s="17" t="n"/>
       <c r="I8" s="14" t="n"/>
       <c r="J8" s="14" t="n"/>
     </row>
@@ -3101,7 +3114,7 @@
       <c r="E9" s="6" t="n"/>
       <c r="F9" s="6" t="n"/>
       <c r="G9" s="6" t="n"/>
-      <c r="H9" s="16" t="n"/>
+      <c r="H9" s="18" t="n"/>
       <c r="I9" s="6" t="n"/>
       <c r="J9" s="6" t="n"/>
     </row>
@@ -3113,7 +3126,7 @@
       <c r="E10" s="14" t="n"/>
       <c r="F10" s="14" t="n"/>
       <c r="G10" s="14" t="n"/>
-      <c r="H10" s="15" t="n"/>
+      <c r="H10" s="17" t="n"/>
       <c r="I10" s="14" t="n"/>
       <c r="J10" s="14" t="n"/>
     </row>
@@ -3125,7 +3138,7 @@
       <c r="E11" s="6" t="n"/>
       <c r="F11" s="6" t="n"/>
       <c r="G11" s="6" t="n"/>
-      <c r="H11" s="16" t="n"/>
+      <c r="H11" s="18" t="n"/>
       <c r="I11" s="6" t="n"/>
       <c r="J11" s="6" t="n"/>
     </row>
@@ -3137,7 +3150,7 @@
       <c r="E12" s="14" t="n"/>
       <c r="F12" s="14" t="n"/>
       <c r="G12" s="14" t="n"/>
-      <c r="H12" s="15" t="n"/>
+      <c r="H12" s="17" t="n"/>
       <c r="I12" s="14" t="n"/>
       <c r="J12" s="14" t="n"/>
     </row>
@@ -3149,7 +3162,7 @@
       <c r="E13" s="6" t="n"/>
       <c r="F13" s="6" t="n"/>
       <c r="G13" s="6" t="n"/>
-      <c r="H13" s="16" t="n"/>
+      <c r="H13" s="18" t="n"/>
       <c r="I13" s="6" t="n"/>
       <c r="J13" s="6" t="n"/>
     </row>
@@ -3161,7 +3174,7 @@
       <c r="E14" s="14" t="n"/>
       <c r="F14" s="14" t="n"/>
       <c r="G14" s="14" t="n"/>
-      <c r="H14" s="15" t="n"/>
+      <c r="H14" s="17" t="n"/>
       <c r="I14" s="14" t="n"/>
       <c r="J14" s="14" t="n"/>
     </row>
@@ -3173,7 +3186,7 @@
       <c r="E15" s="6" t="n"/>
       <c r="F15" s="6" t="n"/>
       <c r="G15" s="6" t="n"/>
-      <c r="H15" s="16" t="n"/>
+      <c r="H15" s="18" t="n"/>
       <c r="I15" s="6" t="n"/>
       <c r="J15" s="6" t="n"/>
     </row>
@@ -3185,7 +3198,7 @@
       <c r="E16" s="14" t="n"/>
       <c r="F16" s="14" t="n"/>
       <c r="G16" s="14" t="n"/>
-      <c r="H16" s="15" t="n"/>
+      <c r="H16" s="17" t="n"/>
       <c r="I16" s="14" t="n"/>
       <c r="J16" s="14" t="n"/>
     </row>
@@ -3197,7 +3210,7 @@
       <c r="E17" s="6" t="n"/>
       <c r="F17" s="6" t="n"/>
       <c r="G17" s="6" t="n"/>
-      <c r="H17" s="16" t="n"/>
+      <c r="H17" s="18" t="n"/>
       <c r="I17" s="6" t="n"/>
       <c r="J17" s="6" t="n"/>
     </row>
@@ -3209,7 +3222,7 @@
       <c r="E18" s="14" t="n"/>
       <c r="F18" s="14" t="n"/>
       <c r="G18" s="14" t="n"/>
-      <c r="H18" s="15" t="n"/>
+      <c r="H18" s="17" t="n"/>
       <c r="I18" s="14" t="n"/>
       <c r="J18" s="14" t="n"/>
     </row>
@@ -3221,7 +3234,7 @@
       <c r="E19" s="6" t="n"/>
       <c r="F19" s="6" t="n"/>
       <c r="G19" s="6" t="n"/>
-      <c r="H19" s="16" t="n"/>
+      <c r="H19" s="18" t="n"/>
       <c r="I19" s="6" t="n"/>
       <c r="J19" s="6" t="n"/>
     </row>
@@ -3233,7 +3246,7 @@
       <c r="E20" s="14" t="n"/>
       <c r="F20" s="14" t="n"/>
       <c r="G20" s="14" t="n"/>
-      <c r="H20" s="15" t="n"/>
+      <c r="H20" s="17" t="n"/>
       <c r="I20" s="14" t="n"/>
       <c r="J20" s="14" t="n"/>
     </row>
@@ -3245,7 +3258,7 @@
       <c r="E21" s="6" t="n"/>
       <c r="F21" s="6" t="n"/>
       <c r="G21" s="6" t="n"/>
-      <c r="H21" s="16" t="n"/>
+      <c r="H21" s="18" t="n"/>
       <c r="I21" s="6" t="n"/>
       <c r="J21" s="6" t="n"/>
     </row>
@@ -3257,7 +3270,7 @@
       <c r="E22" s="14" t="n"/>
       <c r="F22" s="14" t="n"/>
       <c r="G22" s="14" t="n"/>
-      <c r="H22" s="15" t="n"/>
+      <c r="H22" s="17" t="n"/>
       <c r="I22" s="14" t="n"/>
       <c r="J22" s="14" t="n"/>
     </row>
@@ -3269,7 +3282,7 @@
       <c r="E23" s="6" t="n"/>
       <c r="F23" s="6" t="n"/>
       <c r="G23" s="6" t="n"/>
-      <c r="H23" s="16" t="n"/>
+      <c r="H23" s="18" t="n"/>
       <c r="I23" s="6" t="n"/>
       <c r="J23" s="6" t="n"/>
     </row>
@@ -3281,7 +3294,7 @@
       <c r="E24" s="14" t="n"/>
       <c r="F24" s="14" t="n"/>
       <c r="G24" s="14" t="n"/>
-      <c r="H24" s="15" t="n"/>
+      <c r="H24" s="17" t="n"/>
       <c r="I24" s="14" t="n"/>
       <c r="J24" s="14" t="n"/>
     </row>
@@ -3293,7 +3306,7 @@
       <c r="E25" s="6" t="n"/>
       <c r="F25" s="6" t="n"/>
       <c r="G25" s="6" t="n"/>
-      <c r="H25" s="16" t="n"/>
+      <c r="H25" s="18" t="n"/>
       <c r="I25" s="6" t="n"/>
       <c r="J25" s="6" t="n"/>
     </row>
@@ -3305,7 +3318,7 @@
       <c r="E26" s="14" t="n"/>
       <c r="F26" s="14" t="n"/>
       <c r="G26" s="14" t="n"/>
-      <c r="H26" s="15" t="n"/>
+      <c r="H26" s="17" t="n"/>
       <c r="I26" s="14" t="n"/>
       <c r="J26" s="14" t="n"/>
     </row>
@@ -3317,7 +3330,7 @@
       <c r="E27" s="6" t="n"/>
       <c r="F27" s="6" t="n"/>
       <c r="G27" s="6" t="n"/>
-      <c r="H27" s="16" t="n"/>
+      <c r="H27" s="18" t="n"/>
       <c r="I27" s="6" t="n"/>
       <c r="J27" s="6" t="n"/>
     </row>
@@ -3329,7 +3342,7 @@
       <c r="E28" s="14" t="n"/>
       <c r="F28" s="14" t="n"/>
       <c r="G28" s="14" t="n"/>
-      <c r="H28" s="15" t="n"/>
+      <c r="H28" s="17" t="n"/>
       <c r="I28" s="14" t="n"/>
       <c r="J28" s="14" t="n"/>
     </row>
@@ -3341,7 +3354,7 @@
       <c r="E29" s="6" t="n"/>
       <c r="F29" s="6" t="n"/>
       <c r="G29" s="6" t="n"/>
-      <c r="H29" s="16" t="n"/>
+      <c r="H29" s="18" t="n"/>
       <c r="I29" s="6" t="n"/>
       <c r="J29" s="6" t="n"/>
     </row>
@@ -3353,7 +3366,7 @@
       <c r="E30" s="14" t="n"/>
       <c r="F30" s="14" t="n"/>
       <c r="G30" s="14" t="n"/>
-      <c r="H30" s="15" t="n"/>
+      <c r="H30" s="17" t="n"/>
       <c r="I30" s="14" t="n"/>
       <c r="J30" s="14" t="n"/>
     </row>
@@ -3365,7 +3378,7 @@
       <c r="E31" s="6" t="n"/>
       <c r="F31" s="6" t="n"/>
       <c r="G31" s="6" t="n"/>
-      <c r="H31" s="16" t="n"/>
+      <c r="H31" s="18" t="n"/>
       <c r="I31" s="6" t="n"/>
       <c r="J31" s="6" t="n"/>
     </row>
@@ -3377,7 +3390,7 @@
       <c r="E32" s="14" t="n"/>
       <c r="F32" s="14" t="n"/>
       <c r="G32" s="14" t="n"/>
-      <c r="H32" s="15" t="n"/>
+      <c r="H32" s="17" t="n"/>
       <c r="I32" s="14" t="n"/>
       <c r="J32" s="14" t="n"/>
     </row>
@@ -3389,7 +3402,7 @@
       <c r="E33" s="6" t="n"/>
       <c r="F33" s="6" t="n"/>
       <c r="G33" s="6" t="n"/>
-      <c r="H33" s="16" t="n"/>
+      <c r="H33" s="18" t="n"/>
       <c r="I33" s="6" t="n"/>
       <c r="J33" s="6" t="n"/>
     </row>
@@ -3401,7 +3414,7 @@
       <c r="E34" s="14" t="n"/>
       <c r="F34" s="14" t="n"/>
       <c r="G34" s="14" t="n"/>
-      <c r="H34" s="15" t="n"/>
+      <c r="H34" s="17" t="n"/>
       <c r="I34" s="14" t="n"/>
       <c r="J34" s="14" t="n"/>
     </row>
@@ -3413,7 +3426,7 @@
       <c r="E35" s="6" t="n"/>
       <c r="F35" s="6" t="n"/>
       <c r="G35" s="6" t="n"/>
-      <c r="H35" s="16" t="n"/>
+      <c r="H35" s="18" t="n"/>
       <c r="I35" s="6" t="n"/>
       <c r="J35" s="6" t="n"/>
     </row>
@@ -3425,7 +3438,7 @@
       <c r="E36" s="14" t="n"/>
       <c r="F36" s="14" t="n"/>
       <c r="G36" s="14" t="n"/>
-      <c r="H36" s="15" t="n"/>
+      <c r="H36" s="17" t="n"/>
       <c r="I36" s="14" t="n"/>
       <c r="J36" s="14" t="n"/>
     </row>
@@ -3437,7 +3450,7 @@
       <c r="E37" s="6" t="n"/>
       <c r="F37" s="6" t="n"/>
       <c r="G37" s="6" t="n"/>
-      <c r="H37" s="16" t="n"/>
+      <c r="H37" s="18" t="n"/>
       <c r="I37" s="6" t="n"/>
       <c r="J37" s="6" t="n"/>
     </row>
@@ -3449,7 +3462,7 @@
       <c r="E38" s="14" t="n"/>
       <c r="F38" s="14" t="n"/>
       <c r="G38" s="14" t="n"/>
-      <c r="H38" s="15" t="n"/>
+      <c r="H38" s="17" t="n"/>
       <c r="I38" s="14" t="n"/>
       <c r="J38" s="14" t="n"/>
     </row>
@@ -3461,7 +3474,7 @@
       <c r="E39" s="6" t="n"/>
       <c r="F39" s="6" t="n"/>
       <c r="G39" s="6" t="n"/>
-      <c r="H39" s="16" t="n"/>
+      <c r="H39" s="18" t="n"/>
       <c r="I39" s="6" t="n"/>
       <c r="J39" s="6" t="n"/>
     </row>
@@ -3473,7 +3486,7 @@
       <c r="E40" s="14" t="n"/>
       <c r="F40" s="14" t="n"/>
       <c r="G40" s="14" t="n"/>
-      <c r="H40" s="15" t="n"/>
+      <c r="H40" s="17" t="n"/>
       <c r="I40" s="14" t="n"/>
       <c r="J40" s="14" t="n"/>
     </row>
@@ -3485,7 +3498,7 @@
       <c r="E41" s="6" t="n"/>
       <c r="F41" s="6" t="n"/>
       <c r="G41" s="6" t="n"/>
-      <c r="H41" s="16" t="n"/>
+      <c r="H41" s="18" t="n"/>
       <c r="I41" s="6" t="n"/>
       <c r="J41" s="6" t="n"/>
     </row>
@@ -3497,7 +3510,7 @@
       <c r="E42" s="14" t="n"/>
       <c r="F42" s="14" t="n"/>
       <c r="G42" s="14" t="n"/>
-      <c r="H42" s="15" t="n"/>
+      <c r="H42" s="17" t="n"/>
       <c r="I42" s="14" t="n"/>
       <c r="J42" s="14" t="n"/>
     </row>
@@ -3509,7 +3522,7 @@
       <c r="E43" s="6" t="n"/>
       <c r="F43" s="6" t="n"/>
       <c r="G43" s="6" t="n"/>
-      <c r="H43" s="16" t="n"/>
+      <c r="H43" s="18" t="n"/>
       <c r="I43" s="6" t="n"/>
       <c r="J43" s="6" t="n"/>
     </row>
@@ -3608,7 +3621,7 @@
           <t>Rahul Sharma</t>
         </is>
       </c>
-      <c r="D2" s="15" t="n">
+      <c r="D2" s="17" t="n">
         <v>46123</v>
       </c>
       <c r="E2" s="14" t="inlineStr">
@@ -3616,7 +3629,7 @@
           <t>MED-2025-001</t>
         </is>
       </c>
-      <c r="F2" s="15" t="n">
+      <c r="F2" s="17" t="n">
         <v>46488</v>
       </c>
       <c r="G2" s="14">
@@ -3644,7 +3657,7 @@
           <t>Anita Verma</t>
         </is>
       </c>
-      <c r="D3" s="16" t="n">
+      <c r="D3" s="18" t="n">
         <v>45863</v>
       </c>
       <c r="E3" s="6" t="inlineStr">
@@ -3652,7 +3665,7 @@
           <t>MED-2024-045</t>
         </is>
       </c>
-      <c r="F3" s="16" t="n">
+      <c r="F3" s="18" t="n">
         <v>46228</v>
       </c>
       <c r="G3" s="6">
@@ -3674,9 +3687,9 @@
       <c r="A4" s="14" t="n"/>
       <c r="B4" s="14" t="n"/>
       <c r="C4" s="14" t="n"/>
-      <c r="D4" s="15" t="n"/>
+      <c r="D4" s="17" t="n"/>
       <c r="E4" s="14" t="n"/>
-      <c r="F4" s="15" t="n"/>
+      <c r="F4" s="17" t="n"/>
       <c r="G4" s="14">
         <f>IF(F4="","",F4-TODAY())</f>
         <v/>
@@ -3688,9 +3701,9 @@
       <c r="A5" s="6" t="n"/>
       <c r="B5" s="6" t="n"/>
       <c r="C5" s="6" t="n"/>
-      <c r="D5" s="16" t="n"/>
+      <c r="D5" s="18" t="n"/>
       <c r="E5" s="6" t="n"/>
-      <c r="F5" s="16" t="n"/>
+      <c r="F5" s="18" t="n"/>
       <c r="G5" s="6">
         <f>IF(F5="","",F5-TODAY())</f>
         <v/>
@@ -3702,9 +3715,9 @@
       <c r="A6" s="14" t="n"/>
       <c r="B6" s="14" t="n"/>
       <c r="C6" s="14" t="n"/>
-      <c r="D6" s="15" t="n"/>
+      <c r="D6" s="17" t="n"/>
       <c r="E6" s="14" t="n"/>
-      <c r="F6" s="15" t="n"/>
+      <c r="F6" s="17" t="n"/>
       <c r="G6" s="14">
         <f>IF(F6="","",F6-TODAY())</f>
         <v/>
@@ -3716,9 +3729,9 @@
       <c r="A7" s="6" t="n"/>
       <c r="B7" s="6" t="n"/>
       <c r="C7" s="6" t="n"/>
-      <c r="D7" s="16" t="n"/>
+      <c r="D7" s="18" t="n"/>
       <c r="E7" s="6" t="n"/>
-      <c r="F7" s="16" t="n"/>
+      <c r="F7" s="18" t="n"/>
       <c r="G7" s="6">
         <f>IF(F7="","",F7-TODAY())</f>
         <v/>
@@ -3730,9 +3743,9 @@
       <c r="A8" s="14" t="n"/>
       <c r="B8" s="14" t="n"/>
       <c r="C8" s="14" t="n"/>
-      <c r="D8" s="15" t="n"/>
+      <c r="D8" s="17" t="n"/>
       <c r="E8" s="14" t="n"/>
-      <c r="F8" s="15" t="n"/>
+      <c r="F8" s="17" t="n"/>
       <c r="G8" s="14">
         <f>IF(F8="","",F8-TODAY())</f>
         <v/>
@@ -3744,9 +3757,9 @@
       <c r="A9" s="6" t="n"/>
       <c r="B9" s="6" t="n"/>
       <c r="C9" s="6" t="n"/>
-      <c r="D9" s="16" t="n"/>
+      <c r="D9" s="18" t="n"/>
       <c r="E9" s="6" t="n"/>
-      <c r="F9" s="16" t="n"/>
+      <c r="F9" s="18" t="n"/>
       <c r="G9" s="6">
         <f>IF(F9="","",F9-TODAY())</f>
         <v/>
@@ -3758,9 +3771,9 @@
       <c r="A10" s="14" t="n"/>
       <c r="B10" s="14" t="n"/>
       <c r="C10" s="14" t="n"/>
-      <c r="D10" s="15" t="n"/>
+      <c r="D10" s="17" t="n"/>
       <c r="E10" s="14" t="n"/>
-      <c r="F10" s="15" t="n"/>
+      <c r="F10" s="17" t="n"/>
       <c r="G10" s="14">
         <f>IF(F10="","",F10-TODAY())</f>
         <v/>
@@ -3772,9 +3785,9 @@
       <c r="A11" s="6" t="n"/>
       <c r="B11" s="6" t="n"/>
       <c r="C11" s="6" t="n"/>
-      <c r="D11" s="16" t="n"/>
+      <c r="D11" s="18" t="n"/>
       <c r="E11" s="6" t="n"/>
-      <c r="F11" s="16" t="n"/>
+      <c r="F11" s="18" t="n"/>
       <c r="G11" s="6">
         <f>IF(F11="","",F11-TODAY())</f>
         <v/>
@@ -3786,9 +3799,9 @@
       <c r="A12" s="14" t="n"/>
       <c r="B12" s="14" t="n"/>
       <c r="C12" s="14" t="n"/>
-      <c r="D12" s="15" t="n"/>
+      <c r="D12" s="17" t="n"/>
       <c r="E12" s="14" t="n"/>
-      <c r="F12" s="15" t="n"/>
+      <c r="F12" s="17" t="n"/>
       <c r="G12" s="14">
         <f>IF(F12="","",F12-TODAY())</f>
         <v/>
@@ -3800,9 +3813,9 @@
       <c r="A13" s="6" t="n"/>
       <c r="B13" s="6" t="n"/>
       <c r="C13" s="6" t="n"/>
-      <c r="D13" s="16" t="n"/>
+      <c r="D13" s="18" t="n"/>
       <c r="E13" s="6" t="n"/>
-      <c r="F13" s="16" t="n"/>
+      <c r="F13" s="18" t="n"/>
       <c r="G13" s="6">
         <f>IF(F13="","",F13-TODAY())</f>
         <v/>
@@ -3814,9 +3827,9 @@
       <c r="A14" s="14" t="n"/>
       <c r="B14" s="14" t="n"/>
       <c r="C14" s="14" t="n"/>
-      <c r="D14" s="15" t="n"/>
+      <c r="D14" s="17" t="n"/>
       <c r="E14" s="14" t="n"/>
-      <c r="F14" s="15" t="n"/>
+      <c r="F14" s="17" t="n"/>
       <c r="G14" s="14">
         <f>IF(F14="","",F14-TODAY())</f>
         <v/>
@@ -3828,9 +3841,9 @@
       <c r="A15" s="6" t="n"/>
       <c r="B15" s="6" t="n"/>
       <c r="C15" s="6" t="n"/>
-      <c r="D15" s="16" t="n"/>
+      <c r="D15" s="18" t="n"/>
       <c r="E15" s="6" t="n"/>
-      <c r="F15" s="16" t="n"/>
+      <c r="F15" s="18" t="n"/>
       <c r="G15" s="6">
         <f>IF(F15="","",F15-TODAY())</f>
         <v/>
@@ -3842,9 +3855,9 @@
       <c r="A16" s="14" t="n"/>
       <c r="B16" s="14" t="n"/>
       <c r="C16" s="14" t="n"/>
-      <c r="D16" s="15" t="n"/>
+      <c r="D16" s="17" t="n"/>
       <c r="E16" s="14" t="n"/>
-      <c r="F16" s="15" t="n"/>
+      <c r="F16" s="17" t="n"/>
       <c r="G16" s="14">
         <f>IF(F16="","",F16-TODAY())</f>
         <v/>
@@ -3856,9 +3869,9 @@
       <c r="A17" s="6" t="n"/>
       <c r="B17" s="6" t="n"/>
       <c r="C17" s="6" t="n"/>
-      <c r="D17" s="16" t="n"/>
+      <c r="D17" s="18" t="n"/>
       <c r="E17" s="6" t="n"/>
-      <c r="F17" s="16" t="n"/>
+      <c r="F17" s="18" t="n"/>
       <c r="G17" s="6">
         <f>IF(F17="","",F17-TODAY())</f>
         <v/>
@@ -3870,9 +3883,9 @@
       <c r="A18" s="14" t="n"/>
       <c r="B18" s="14" t="n"/>
       <c r="C18" s="14" t="n"/>
-      <c r="D18" s="15" t="n"/>
+      <c r="D18" s="17" t="n"/>
       <c r="E18" s="14" t="n"/>
-      <c r="F18" s="15" t="n"/>
+      <c r="F18" s="17" t="n"/>
       <c r="G18" s="14">
         <f>IF(F18="","",F18-TODAY())</f>
         <v/>
@@ -3884,9 +3897,9 @@
       <c r="A19" s="6" t="n"/>
       <c r="B19" s="6" t="n"/>
       <c r="C19" s="6" t="n"/>
-      <c r="D19" s="16" t="n"/>
+      <c r="D19" s="18" t="n"/>
       <c r="E19" s="6" t="n"/>
-      <c r="F19" s="16" t="n"/>
+      <c r="F19" s="18" t="n"/>
       <c r="G19" s="6">
         <f>IF(F19="","",F19-TODAY())</f>
         <v/>
@@ -3898,9 +3911,9 @@
       <c r="A20" s="14" t="n"/>
       <c r="B20" s="14" t="n"/>
       <c r="C20" s="14" t="n"/>
-      <c r="D20" s="15" t="n"/>
+      <c r="D20" s="17" t="n"/>
       <c r="E20" s="14" t="n"/>
-      <c r="F20" s="15" t="n"/>
+      <c r="F20" s="17" t="n"/>
       <c r="G20" s="14">
         <f>IF(F20="","",F20-TODAY())</f>
         <v/>
@@ -3912,9 +3925,9 @@
       <c r="A21" s="6" t="n"/>
       <c r="B21" s="6" t="n"/>
       <c r="C21" s="6" t="n"/>
-      <c r="D21" s="16" t="n"/>
+      <c r="D21" s="18" t="n"/>
       <c r="E21" s="6" t="n"/>
-      <c r="F21" s="16" t="n"/>
+      <c r="F21" s="18" t="n"/>
       <c r="G21" s="6">
         <f>IF(F21="","",F21-TODAY())</f>
         <v/>
@@ -3926,9 +3939,9 @@
       <c r="A22" s="14" t="n"/>
       <c r="B22" s="14" t="n"/>
       <c r="C22" s="14" t="n"/>
-      <c r="D22" s="15" t="n"/>
+      <c r="D22" s="17" t="n"/>
       <c r="E22" s="14" t="n"/>
-      <c r="F22" s="15" t="n"/>
+      <c r="F22" s="17" t="n"/>
       <c r="G22" s="14">
         <f>IF(F22="","",F22-TODAY())</f>
         <v/>
@@ -3940,9 +3953,9 @@
       <c r="A23" s="6" t="n"/>
       <c r="B23" s="6" t="n"/>
       <c r="C23" s="6" t="n"/>
-      <c r="D23" s="16" t="n"/>
+      <c r="D23" s="18" t="n"/>
       <c r="E23" s="6" t="n"/>
-      <c r="F23" s="16" t="n"/>
+      <c r="F23" s="18" t="n"/>
       <c r="G23" s="6">
         <f>IF(F23="","",F23-TODAY())</f>
         <v/>
@@ -3954,9 +3967,9 @@
       <c r="A24" s="14" t="n"/>
       <c r="B24" s="14" t="n"/>
       <c r="C24" s="14" t="n"/>
-      <c r="D24" s="15" t="n"/>
+      <c r="D24" s="17" t="n"/>
       <c r="E24" s="14" t="n"/>
-      <c r="F24" s="15" t="n"/>
+      <c r="F24" s="17" t="n"/>
       <c r="G24" s="14">
         <f>IF(F24="","",F24-TODAY())</f>
         <v/>
@@ -3968,9 +3981,9 @@
       <c r="A25" s="6" t="n"/>
       <c r="B25" s="6" t="n"/>
       <c r="C25" s="6" t="n"/>
-      <c r="D25" s="16" t="n"/>
+      <c r="D25" s="18" t="n"/>
       <c r="E25" s="6" t="n"/>
-      <c r="F25" s="16" t="n"/>
+      <c r="F25" s="18" t="n"/>
       <c r="G25" s="6">
         <f>IF(F25="","",F25-TODAY())</f>
         <v/>
@@ -3982,9 +3995,9 @@
       <c r="A26" s="14" t="n"/>
       <c r="B26" s="14" t="n"/>
       <c r="C26" s="14" t="n"/>
-      <c r="D26" s="15" t="n"/>
+      <c r="D26" s="17" t="n"/>
       <c r="E26" s="14" t="n"/>
-      <c r="F26" s="15" t="n"/>
+      <c r="F26" s="17" t="n"/>
       <c r="G26" s="14">
         <f>IF(F26="","",F26-TODAY())</f>
         <v/>
@@ -3996,9 +4009,9 @@
       <c r="A27" s="6" t="n"/>
       <c r="B27" s="6" t="n"/>
       <c r="C27" s="6" t="n"/>
-      <c r="D27" s="16" t="n"/>
+      <c r="D27" s="18" t="n"/>
       <c r="E27" s="6" t="n"/>
-      <c r="F27" s="16" t="n"/>
+      <c r="F27" s="18" t="n"/>
       <c r="G27" s="6">
         <f>IF(F27="","",F27-TODAY())</f>
         <v/>
@@ -4010,9 +4023,9 @@
       <c r="A28" s="14" t="n"/>
       <c r="B28" s="14" t="n"/>
       <c r="C28" s="14" t="n"/>
-      <c r="D28" s="15" t="n"/>
+      <c r="D28" s="17" t="n"/>
       <c r="E28" s="14" t="n"/>
-      <c r="F28" s="15" t="n"/>
+      <c r="F28" s="17" t="n"/>
       <c r="G28" s="14">
         <f>IF(F28="","",F28-TODAY())</f>
         <v/>
@@ -4024,9 +4037,9 @@
       <c r="A29" s="6" t="n"/>
       <c r="B29" s="6" t="n"/>
       <c r="C29" s="6" t="n"/>
-      <c r="D29" s="16" t="n"/>
+      <c r="D29" s="18" t="n"/>
       <c r="E29" s="6" t="n"/>
-      <c r="F29" s="16" t="n"/>
+      <c r="F29" s="18" t="n"/>
       <c r="G29" s="6">
         <f>IF(F29="","",F29-TODAY())</f>
         <v/>
@@ -4038,9 +4051,9 @@
       <c r="A30" s="14" t="n"/>
       <c r="B30" s="14" t="n"/>
       <c r="C30" s="14" t="n"/>
-      <c r="D30" s="15" t="n"/>
+      <c r="D30" s="17" t="n"/>
       <c r="E30" s="14" t="n"/>
-      <c r="F30" s="15" t="n"/>
+      <c r="F30" s="17" t="n"/>
       <c r="G30" s="14">
         <f>IF(F30="","",F30-TODAY())</f>
         <v/>
@@ -4052,9 +4065,9 @@
       <c r="A31" s="6" t="n"/>
       <c r="B31" s="6" t="n"/>
       <c r="C31" s="6" t="n"/>
-      <c r="D31" s="16" t="n"/>
+      <c r="D31" s="18" t="n"/>
       <c r="E31" s="6" t="n"/>
-      <c r="F31" s="16" t="n"/>
+      <c r="F31" s="18" t="n"/>
       <c r="G31" s="6">
         <f>IF(F31="","",F31-TODAY())</f>
         <v/>
@@ -4066,9 +4079,9 @@
       <c r="A32" s="14" t="n"/>
       <c r="B32" s="14" t="n"/>
       <c r="C32" s="14" t="n"/>
-      <c r="D32" s="15" t="n"/>
+      <c r="D32" s="17" t="n"/>
       <c r="E32" s="14" t="n"/>
-      <c r="F32" s="15" t="n"/>
+      <c r="F32" s="17" t="n"/>
       <c r="G32" s="14">
         <f>IF(F32="","",F32-TODAY())</f>
         <v/>
@@ -4080,9 +4093,9 @@
       <c r="A33" s="6" t="n"/>
       <c r="B33" s="6" t="n"/>
       <c r="C33" s="6" t="n"/>
-      <c r="D33" s="16" t="n"/>
+      <c r="D33" s="18" t="n"/>
       <c r="E33" s="6" t="n"/>
-      <c r="F33" s="16" t="n"/>
+      <c r="F33" s="18" t="n"/>
       <c r="G33" s="6">
         <f>IF(F33="","",F33-TODAY())</f>
         <v/>
@@ -4094,9 +4107,9 @@
       <c r="A34" s="14" t="n"/>
       <c r="B34" s="14" t="n"/>
       <c r="C34" s="14" t="n"/>
-      <c r="D34" s="15" t="n"/>
+      <c r="D34" s="17" t="n"/>
       <c r="E34" s="14" t="n"/>
-      <c r="F34" s="15" t="n"/>
+      <c r="F34" s="17" t="n"/>
       <c r="G34" s="14">
         <f>IF(F34="","",F34-TODAY())</f>
         <v/>
@@ -4108,9 +4121,9 @@
       <c r="A35" s="6" t="n"/>
       <c r="B35" s="6" t="n"/>
       <c r="C35" s="6" t="n"/>
-      <c r="D35" s="16" t="n"/>
+      <c r="D35" s="18" t="n"/>
       <c r="E35" s="6" t="n"/>
-      <c r="F35" s="16" t="n"/>
+      <c r="F35" s="18" t="n"/>
       <c r="G35" s="6">
         <f>IF(F35="","",F35-TODAY())</f>
         <v/>
@@ -4122,9 +4135,9 @@
       <c r="A36" s="14" t="n"/>
       <c r="B36" s="14" t="n"/>
       <c r="C36" s="14" t="n"/>
-      <c r="D36" s="15" t="n"/>
+      <c r="D36" s="17" t="n"/>
       <c r="E36" s="14" t="n"/>
-      <c r="F36" s="15" t="n"/>
+      <c r="F36" s="17" t="n"/>
       <c r="G36" s="14">
         <f>IF(F36="","",F36-TODAY())</f>
         <v/>
@@ -4136,9 +4149,9 @@
       <c r="A37" s="6" t="n"/>
       <c r="B37" s="6" t="n"/>
       <c r="C37" s="6" t="n"/>
-      <c r="D37" s="16" t="n"/>
+      <c r="D37" s="18" t="n"/>
       <c r="E37" s="6" t="n"/>
-      <c r="F37" s="16" t="n"/>
+      <c r="F37" s="18" t="n"/>
       <c r="G37" s="6">
         <f>IF(F37="","",F37-TODAY())</f>
         <v/>
@@ -4150,9 +4163,9 @@
       <c r="A38" s="14" t="n"/>
       <c r="B38" s="14" t="n"/>
       <c r="C38" s="14" t="n"/>
-      <c r="D38" s="15" t="n"/>
+      <c r="D38" s="17" t="n"/>
       <c r="E38" s="14" t="n"/>
-      <c r="F38" s="15" t="n"/>
+      <c r="F38" s="17" t="n"/>
       <c r="G38" s="14">
         <f>IF(F38="","",F38-TODAY())</f>
         <v/>
@@ -4164,9 +4177,9 @@
       <c r="A39" s="6" t="n"/>
       <c r="B39" s="6" t="n"/>
       <c r="C39" s="6" t="n"/>
-      <c r="D39" s="16" t="n"/>
+      <c r="D39" s="18" t="n"/>
       <c r="E39" s="6" t="n"/>
-      <c r="F39" s="16" t="n"/>
+      <c r="F39" s="18" t="n"/>
       <c r="G39" s="6">
         <f>IF(F39="","",F39-TODAY())</f>
         <v/>
@@ -4178,9 +4191,9 @@
       <c r="A40" s="14" t="n"/>
       <c r="B40" s="14" t="n"/>
       <c r="C40" s="14" t="n"/>
-      <c r="D40" s="15" t="n"/>
+      <c r="D40" s="17" t="n"/>
       <c r="E40" s="14" t="n"/>
-      <c r="F40" s="15" t="n"/>
+      <c r="F40" s="17" t="n"/>
       <c r="G40" s="14">
         <f>IF(F40="","",F40-TODAY())</f>
         <v/>
@@ -4192,9 +4205,9 @@
       <c r="A41" s="6" t="n"/>
       <c r="B41" s="6" t="n"/>
       <c r="C41" s="6" t="n"/>
-      <c r="D41" s="16" t="n"/>
+      <c r="D41" s="18" t="n"/>
       <c r="E41" s="6" t="n"/>
-      <c r="F41" s="16" t="n"/>
+      <c r="F41" s="18" t="n"/>
       <c r="G41" s="6">
         <f>IF(F41="","",F41-TODAY())</f>
         <v/>
@@ -4206,9 +4219,9 @@
       <c r="A42" s="14" t="n"/>
       <c r="B42" s="14" t="n"/>
       <c r="C42" s="14" t="n"/>
-      <c r="D42" s="15" t="n"/>
+      <c r="D42" s="17" t="n"/>
       <c r="E42" s="14" t="n"/>
-      <c r="F42" s="15" t="n"/>
+      <c r="F42" s="17" t="n"/>
       <c r="G42" s="14">
         <f>IF(F42="","",F42-TODAY())</f>
         <v/>
@@ -4220,9 +4233,9 @@
       <c r="A43" s="6" t="n"/>
       <c r="B43" s="6" t="n"/>
       <c r="C43" s="6" t="n"/>
-      <c r="D43" s="16" t="n"/>
+      <c r="D43" s="18" t="n"/>
       <c r="E43" s="6" t="n"/>
-      <c r="F43" s="16" t="n"/>
+      <c r="F43" s="18" t="n"/>
       <c r="G43" s="6">
         <f>IF(F43="","",F43-TODAY())</f>
         <v/>
@@ -4339,7 +4352,7 @@
           <t>Rahul Sharma</t>
         </is>
       </c>
-      <c r="D2" s="15" t="n">
+      <c r="D2" s="17" t="n">
         <v>46073</v>
       </c>
       <c r="E2" s="14" t="inlineStr">
@@ -4352,7 +4365,7 @@
           <t>MG Road PS</t>
         </is>
       </c>
-      <c r="G2" s="15" t="n">
+      <c r="G2" s="17" t="n">
         <v>46803</v>
       </c>
       <c r="H2" s="14">
@@ -4380,7 +4393,7 @@
           <t>Anita Verma</t>
         </is>
       </c>
-      <c r="D3" s="16" t="n">
+      <c r="D3" s="18" t="n">
         <v>46203</v>
       </c>
       <c r="E3" s="6" t="inlineStr">
@@ -4393,7 +4406,7 @@
           <t>MG Road PS</t>
         </is>
       </c>
-      <c r="G3" s="16" t="n">
+      <c r="G3" s="18" t="n">
         <v>46933</v>
       </c>
       <c r="H3" s="6">
@@ -4411,10 +4424,10 @@
       <c r="A4" s="14" t="n"/>
       <c r="B4" s="14" t="n"/>
       <c r="C4" s="14" t="n"/>
-      <c r="D4" s="15" t="n"/>
+      <c r="D4" s="17" t="n"/>
       <c r="E4" s="14" t="n"/>
       <c r="F4" s="14" t="n"/>
-      <c r="G4" s="15" t="n"/>
+      <c r="G4" s="17" t="n"/>
       <c r="H4" s="14">
         <f>IF(G4="","",G4-TODAY())</f>
         <v/>
@@ -4426,10 +4439,10 @@
       <c r="A5" s="6" t="n"/>
       <c r="B5" s="6" t="n"/>
       <c r="C5" s="6" t="n"/>
-      <c r="D5" s="16" t="n"/>
+      <c r="D5" s="18" t="n"/>
       <c r="E5" s="6" t="n"/>
       <c r="F5" s="6" t="n"/>
-      <c r="G5" s="16" t="n"/>
+      <c r="G5" s="18" t="n"/>
       <c r="H5" s="6">
         <f>IF(G5="","",G5-TODAY())</f>
         <v/>
@@ -4441,10 +4454,10 @@
       <c r="A6" s="14" t="n"/>
       <c r="B6" s="14" t="n"/>
       <c r="C6" s="14" t="n"/>
-      <c r="D6" s="15" t="n"/>
+      <c r="D6" s="17" t="n"/>
       <c r="E6" s="14" t="n"/>
       <c r="F6" s="14" t="n"/>
-      <c r="G6" s="15" t="n"/>
+      <c r="G6" s="17" t="n"/>
       <c r="H6" s="14">
         <f>IF(G6="","",G6-TODAY())</f>
         <v/>
@@ -4456,10 +4469,10 @@
       <c r="A7" s="6" t="n"/>
       <c r="B7" s="6" t="n"/>
       <c r="C7" s="6" t="n"/>
-      <c r="D7" s="16" t="n"/>
+      <c r="D7" s="18" t="n"/>
       <c r="E7" s="6" t="n"/>
       <c r="F7" s="6" t="n"/>
-      <c r="G7" s="16" t="n"/>
+      <c r="G7" s="18" t="n"/>
       <c r="H7" s="6">
         <f>IF(G7="","",G7-TODAY())</f>
         <v/>
@@ -4471,10 +4484,10 @@
       <c r="A8" s="14" t="n"/>
       <c r="B8" s="14" t="n"/>
       <c r="C8" s="14" t="n"/>
-      <c r="D8" s="15" t="n"/>
+      <c r="D8" s="17" t="n"/>
       <c r="E8" s="14" t="n"/>
       <c r="F8" s="14" t="n"/>
-      <c r="G8" s="15" t="n"/>
+      <c r="G8" s="17" t="n"/>
       <c r="H8" s="14">
         <f>IF(G8="","",G8-TODAY())</f>
         <v/>
@@ -4486,10 +4499,10 @@
       <c r="A9" s="6" t="n"/>
       <c r="B9" s="6" t="n"/>
       <c r="C9" s="6" t="n"/>
-      <c r="D9" s="16" t="n"/>
+      <c r="D9" s="18" t="n"/>
       <c r="E9" s="6" t="n"/>
       <c r="F9" s="6" t="n"/>
-      <c r="G9" s="16" t="n"/>
+      <c r="G9" s="18" t="n"/>
       <c r="H9" s="6">
         <f>IF(G9="","",G9-TODAY())</f>
         <v/>
@@ -4501,10 +4514,10 @@
       <c r="A10" s="14" t="n"/>
       <c r="B10" s="14" t="n"/>
       <c r="C10" s="14" t="n"/>
-      <c r="D10" s="15" t="n"/>
+      <c r="D10" s="17" t="n"/>
       <c r="E10" s="14" t="n"/>
       <c r="F10" s="14" t="n"/>
-      <c r="G10" s="15" t="n"/>
+      <c r="G10" s="17" t="n"/>
       <c r="H10" s="14">
         <f>IF(G10="","",G10-TODAY())</f>
         <v/>
@@ -4516,10 +4529,10 @@
       <c r="A11" s="6" t="n"/>
       <c r="B11" s="6" t="n"/>
       <c r="C11" s="6" t="n"/>
-      <c r="D11" s="16" t="n"/>
+      <c r="D11" s="18" t="n"/>
       <c r="E11" s="6" t="n"/>
       <c r="F11" s="6" t="n"/>
-      <c r="G11" s="16" t="n"/>
+      <c r="G11" s="18" t="n"/>
       <c r="H11" s="6">
         <f>IF(G11="","",G11-TODAY())</f>
         <v/>
@@ -4531,10 +4544,10 @@
       <c r="A12" s="14" t="n"/>
       <c r="B12" s="14" t="n"/>
       <c r="C12" s="14" t="n"/>
-      <c r="D12" s="15" t="n"/>
+      <c r="D12" s="17" t="n"/>
       <c r="E12" s="14" t="n"/>
       <c r="F12" s="14" t="n"/>
-      <c r="G12" s="15" t="n"/>
+      <c r="G12" s="17" t="n"/>
       <c r="H12" s="14">
         <f>IF(G12="","",G12-TODAY())</f>
         <v/>
@@ -4546,10 +4559,10 @@
       <c r="A13" s="6" t="n"/>
       <c r="B13" s="6" t="n"/>
       <c r="C13" s="6" t="n"/>
-      <c r="D13" s="16" t="n"/>
+      <c r="D13" s="18" t="n"/>
       <c r="E13" s="6" t="n"/>
       <c r="F13" s="6" t="n"/>
-      <c r="G13" s="16" t="n"/>
+      <c r="G13" s="18" t="n"/>
       <c r="H13" s="6">
         <f>IF(G13="","",G13-TODAY())</f>
         <v/>
@@ -4561,10 +4574,10 @@
       <c r="A14" s="14" t="n"/>
       <c r="B14" s="14" t="n"/>
       <c r="C14" s="14" t="n"/>
-      <c r="D14" s="15" t="n"/>
+      <c r="D14" s="17" t="n"/>
       <c r="E14" s="14" t="n"/>
       <c r="F14" s="14" t="n"/>
-      <c r="G14" s="15" t="n"/>
+      <c r="G14" s="17" t="n"/>
       <c r="H14" s="14">
         <f>IF(G14="","",G14-TODAY())</f>
         <v/>
@@ -4576,10 +4589,10 @@
       <c r="A15" s="6" t="n"/>
       <c r="B15" s="6" t="n"/>
       <c r="C15" s="6" t="n"/>
-      <c r="D15" s="16" t="n"/>
+      <c r="D15" s="18" t="n"/>
       <c r="E15" s="6" t="n"/>
       <c r="F15" s="6" t="n"/>
-      <c r="G15" s="16" t="n"/>
+      <c r="G15" s="18" t="n"/>
       <c r="H15" s="6">
         <f>IF(G15="","",G15-TODAY())</f>
         <v/>
@@ -4591,10 +4604,10 @@
       <c r="A16" s="14" t="n"/>
       <c r="B16" s="14" t="n"/>
       <c r="C16" s="14" t="n"/>
-      <c r="D16" s="15" t="n"/>
+      <c r="D16" s="17" t="n"/>
       <c r="E16" s="14" t="n"/>
       <c r="F16" s="14" t="n"/>
-      <c r="G16" s="15" t="n"/>
+      <c r="G16" s="17" t="n"/>
       <c r="H16" s="14">
         <f>IF(G16="","",G16-TODAY())</f>
         <v/>
@@ -4606,10 +4619,10 @@
       <c r="A17" s="6" t="n"/>
       <c r="B17" s="6" t="n"/>
       <c r="C17" s="6" t="n"/>
-      <c r="D17" s="16" t="n"/>
+      <c r="D17" s="18" t="n"/>
       <c r="E17" s="6" t="n"/>
       <c r="F17" s="6" t="n"/>
-      <c r="G17" s="16" t="n"/>
+      <c r="G17" s="18" t="n"/>
       <c r="H17" s="6">
         <f>IF(G17="","",G17-TODAY())</f>
         <v/>
@@ -4621,10 +4634,10 @@
       <c r="A18" s="14" t="n"/>
       <c r="B18" s="14" t="n"/>
       <c r="C18" s="14" t="n"/>
-      <c r="D18" s="15" t="n"/>
+      <c r="D18" s="17" t="n"/>
       <c r="E18" s="14" t="n"/>
       <c r="F18" s="14" t="n"/>
-      <c r="G18" s="15" t="n"/>
+      <c r="G18" s="17" t="n"/>
       <c r="H18" s="14">
         <f>IF(G18="","",G18-TODAY())</f>
         <v/>
@@ -4636,10 +4649,10 @@
       <c r="A19" s="6" t="n"/>
       <c r="B19" s="6" t="n"/>
       <c r="C19" s="6" t="n"/>
-      <c r="D19" s="16" t="n"/>
+      <c r="D19" s="18" t="n"/>
       <c r="E19" s="6" t="n"/>
       <c r="F19" s="6" t="n"/>
-      <c r="G19" s="16" t="n"/>
+      <c r="G19" s="18" t="n"/>
       <c r="H19" s="6">
         <f>IF(G19="","",G19-TODAY())</f>
         <v/>
@@ -4651,10 +4664,10 @@
       <c r="A20" s="14" t="n"/>
       <c r="B20" s="14" t="n"/>
       <c r="C20" s="14" t="n"/>
-      <c r="D20" s="15" t="n"/>
+      <c r="D20" s="17" t="n"/>
       <c r="E20" s="14" t="n"/>
       <c r="F20" s="14" t="n"/>
-      <c r="G20" s="15" t="n"/>
+      <c r="G20" s="17" t="n"/>
       <c r="H20" s="14">
         <f>IF(G20="","",G20-TODAY())</f>
         <v/>
@@ -4666,10 +4679,10 @@
       <c r="A21" s="6" t="n"/>
       <c r="B21" s="6" t="n"/>
       <c r="C21" s="6" t="n"/>
-      <c r="D21" s="16" t="n"/>
+      <c r="D21" s="18" t="n"/>
       <c r="E21" s="6" t="n"/>
       <c r="F21" s="6" t="n"/>
-      <c r="G21" s="16" t="n"/>
+      <c r="G21" s="18" t="n"/>
       <c r="H21" s="6">
         <f>IF(G21="","",G21-TODAY())</f>
         <v/>
@@ -4681,10 +4694,10 @@
       <c r="A22" s="14" t="n"/>
       <c r="B22" s="14" t="n"/>
       <c r="C22" s="14" t="n"/>
-      <c r="D22" s="15" t="n"/>
+      <c r="D22" s="17" t="n"/>
       <c r="E22" s="14" t="n"/>
       <c r="F22" s="14" t="n"/>
-      <c r="G22" s="15" t="n"/>
+      <c r="G22" s="17" t="n"/>
       <c r="H22" s="14">
         <f>IF(G22="","",G22-TODAY())</f>
         <v/>
@@ -4696,10 +4709,10 @@
       <c r="A23" s="6" t="n"/>
       <c r="B23" s="6" t="n"/>
       <c r="C23" s="6" t="n"/>
-      <c r="D23" s="16" t="n"/>
+      <c r="D23" s="18" t="n"/>
       <c r="E23" s="6" t="n"/>
       <c r="F23" s="6" t="n"/>
-      <c r="G23" s="16" t="n"/>
+      <c r="G23" s="18" t="n"/>
       <c r="H23" s="6">
         <f>IF(G23="","",G23-TODAY())</f>
         <v/>
@@ -4711,10 +4724,10 @@
       <c r="A24" s="14" t="n"/>
       <c r="B24" s="14" t="n"/>
       <c r="C24" s="14" t="n"/>
-      <c r="D24" s="15" t="n"/>
+      <c r="D24" s="17" t="n"/>
       <c r="E24" s="14" t="n"/>
       <c r="F24" s="14" t="n"/>
-      <c r="G24" s="15" t="n"/>
+      <c r="G24" s="17" t="n"/>
       <c r="H24" s="14">
         <f>IF(G24="","",G24-TODAY())</f>
         <v/>
@@ -4726,10 +4739,10 @@
       <c r="A25" s="6" t="n"/>
       <c r="B25" s="6" t="n"/>
       <c r="C25" s="6" t="n"/>
-      <c r="D25" s="16" t="n"/>
+      <c r="D25" s="18" t="n"/>
       <c r="E25" s="6" t="n"/>
       <c r="F25" s="6" t="n"/>
-      <c r="G25" s="16" t="n"/>
+      <c r="G25" s="18" t="n"/>
       <c r="H25" s="6">
         <f>IF(G25="","",G25-TODAY())</f>
         <v/>
@@ -4741,10 +4754,10 @@
       <c r="A26" s="14" t="n"/>
       <c r="B26" s="14" t="n"/>
       <c r="C26" s="14" t="n"/>
-      <c r="D26" s="15" t="n"/>
+      <c r="D26" s="17" t="n"/>
       <c r="E26" s="14" t="n"/>
       <c r="F26" s="14" t="n"/>
-      <c r="G26" s="15" t="n"/>
+      <c r="G26" s="17" t="n"/>
       <c r="H26" s="14">
         <f>IF(G26="","",G26-TODAY())</f>
         <v/>
@@ -4756,10 +4769,10 @@
       <c r="A27" s="6" t="n"/>
       <c r="B27" s="6" t="n"/>
       <c r="C27" s="6" t="n"/>
-      <c r="D27" s="16" t="n"/>
+      <c r="D27" s="18" t="n"/>
       <c r="E27" s="6" t="n"/>
       <c r="F27" s="6" t="n"/>
-      <c r="G27" s="16" t="n"/>
+      <c r="G27" s="18" t="n"/>
       <c r="H27" s="6">
         <f>IF(G27="","",G27-TODAY())</f>
         <v/>
@@ -4771,10 +4784,10 @@
       <c r="A28" s="14" t="n"/>
       <c r="B28" s="14" t="n"/>
       <c r="C28" s="14" t="n"/>
-      <c r="D28" s="15" t="n"/>
+      <c r="D28" s="17" t="n"/>
       <c r="E28" s="14" t="n"/>
       <c r="F28" s="14" t="n"/>
-      <c r="G28" s="15" t="n"/>
+      <c r="G28" s="17" t="n"/>
       <c r="H28" s="14">
         <f>IF(G28="","",G28-TODAY())</f>
         <v/>
@@ -4786,10 +4799,10 @@
       <c r="A29" s="6" t="n"/>
       <c r="B29" s="6" t="n"/>
       <c r="C29" s="6" t="n"/>
-      <c r="D29" s="16" t="n"/>
+      <c r="D29" s="18" t="n"/>
       <c r="E29" s="6" t="n"/>
       <c r="F29" s="6" t="n"/>
-      <c r="G29" s="16" t="n"/>
+      <c r="G29" s="18" t="n"/>
       <c r="H29" s="6">
         <f>IF(G29="","",G29-TODAY())</f>
         <v/>
@@ -4801,10 +4814,10 @@
       <c r="A30" s="14" t="n"/>
       <c r="B30" s="14" t="n"/>
       <c r="C30" s="14" t="n"/>
-      <c r="D30" s="15" t="n"/>
+      <c r="D30" s="17" t="n"/>
       <c r="E30" s="14" t="n"/>
       <c r="F30" s="14" t="n"/>
-      <c r="G30" s="15" t="n"/>
+      <c r="G30" s="17" t="n"/>
       <c r="H30" s="14">
         <f>IF(G30="","",G30-TODAY())</f>
         <v/>
@@ -4816,10 +4829,10 @@
       <c r="A31" s="6" t="n"/>
       <c r="B31" s="6" t="n"/>
       <c r="C31" s="6" t="n"/>
-      <c r="D31" s="16" t="n"/>
+      <c r="D31" s="18" t="n"/>
       <c r="E31" s="6" t="n"/>
       <c r="F31" s="6" t="n"/>
-      <c r="G31" s="16" t="n"/>
+      <c r="G31" s="18" t="n"/>
       <c r="H31" s="6">
         <f>IF(G31="","",G31-TODAY())</f>
         <v/>
@@ -4831,10 +4844,10 @@
       <c r="A32" s="14" t="n"/>
       <c r="B32" s="14" t="n"/>
       <c r="C32" s="14" t="n"/>
-      <c r="D32" s="15" t="n"/>
+      <c r="D32" s="17" t="n"/>
       <c r="E32" s="14" t="n"/>
       <c r="F32" s="14" t="n"/>
-      <c r="G32" s="15" t="n"/>
+      <c r="G32" s="17" t="n"/>
       <c r="H32" s="14">
         <f>IF(G32="","",G32-TODAY())</f>
         <v/>
@@ -4846,10 +4859,10 @@
       <c r="A33" s="6" t="n"/>
       <c r="B33" s="6" t="n"/>
       <c r="C33" s="6" t="n"/>
-      <c r="D33" s="16" t="n"/>
+      <c r="D33" s="18" t="n"/>
       <c r="E33" s="6" t="n"/>
       <c r="F33" s="6" t="n"/>
-      <c r="G33" s="16" t="n"/>
+      <c r="G33" s="18" t="n"/>
       <c r="H33" s="6">
         <f>IF(G33="","",G33-TODAY())</f>
         <v/>
@@ -4861,10 +4874,10 @@
       <c r="A34" s="14" t="n"/>
       <c r="B34" s="14" t="n"/>
       <c r="C34" s="14" t="n"/>
-      <c r="D34" s="15" t="n"/>
+      <c r="D34" s="17" t="n"/>
       <c r="E34" s="14" t="n"/>
       <c r="F34" s="14" t="n"/>
-      <c r="G34" s="15" t="n"/>
+      <c r="G34" s="17" t="n"/>
       <c r="H34" s="14">
         <f>IF(G34="","",G34-TODAY())</f>
         <v/>
@@ -4876,10 +4889,10 @@
       <c r="A35" s="6" t="n"/>
       <c r="B35" s="6" t="n"/>
       <c r="C35" s="6" t="n"/>
-      <c r="D35" s="16" t="n"/>
+      <c r="D35" s="18" t="n"/>
       <c r="E35" s="6" t="n"/>
       <c r="F35" s="6" t="n"/>
-      <c r="G35" s="16" t="n"/>
+      <c r="G35" s="18" t="n"/>
       <c r="H35" s="6">
         <f>IF(G35="","",G35-TODAY())</f>
         <v/>
@@ -4891,10 +4904,10 @@
       <c r="A36" s="14" t="n"/>
       <c r="B36" s="14" t="n"/>
       <c r="C36" s="14" t="n"/>
-      <c r="D36" s="15" t="n"/>
+      <c r="D36" s="17" t="n"/>
       <c r="E36" s="14" t="n"/>
       <c r="F36" s="14" t="n"/>
-      <c r="G36" s="15" t="n"/>
+      <c r="G36" s="17" t="n"/>
       <c r="H36" s="14">
         <f>IF(G36="","",G36-TODAY())</f>
         <v/>
@@ -4906,10 +4919,10 @@
       <c r="A37" s="6" t="n"/>
       <c r="B37" s="6" t="n"/>
       <c r="C37" s="6" t="n"/>
-      <c r="D37" s="16" t="n"/>
+      <c r="D37" s="18" t="n"/>
       <c r="E37" s="6" t="n"/>
       <c r="F37" s="6" t="n"/>
-      <c r="G37" s="16" t="n"/>
+      <c r="G37" s="18" t="n"/>
       <c r="H37" s="6">
         <f>IF(G37="","",G37-TODAY())</f>
         <v/>
@@ -4921,10 +4934,10 @@
       <c r="A38" s="14" t="n"/>
       <c r="B38" s="14" t="n"/>
       <c r="C38" s="14" t="n"/>
-      <c r="D38" s="15" t="n"/>
+      <c r="D38" s="17" t="n"/>
       <c r="E38" s="14" t="n"/>
       <c r="F38" s="14" t="n"/>
-      <c r="G38" s="15" t="n"/>
+      <c r="G38" s="17" t="n"/>
       <c r="H38" s="14">
         <f>IF(G38="","",G38-TODAY())</f>
         <v/>
@@ -4936,10 +4949,10 @@
       <c r="A39" s="6" t="n"/>
       <c r="B39" s="6" t="n"/>
       <c r="C39" s="6" t="n"/>
-      <c r="D39" s="16" t="n"/>
+      <c r="D39" s="18" t="n"/>
       <c r="E39" s="6" t="n"/>
       <c r="F39" s="6" t="n"/>
-      <c r="G39" s="16" t="n"/>
+      <c r="G39" s="18" t="n"/>
       <c r="H39" s="6">
         <f>IF(G39="","",G39-TODAY())</f>
         <v/>
@@ -4951,10 +4964,10 @@
       <c r="A40" s="14" t="n"/>
       <c r="B40" s="14" t="n"/>
       <c r="C40" s="14" t="n"/>
-      <c r="D40" s="15" t="n"/>
+      <c r="D40" s="17" t="n"/>
       <c r="E40" s="14" t="n"/>
       <c r="F40" s="14" t="n"/>
-      <c r="G40" s="15" t="n"/>
+      <c r="G40" s="17" t="n"/>
       <c r="H40" s="14">
         <f>IF(G40="","",G40-TODAY())</f>
         <v/>
@@ -4966,10 +4979,10 @@
       <c r="A41" s="6" t="n"/>
       <c r="B41" s="6" t="n"/>
       <c r="C41" s="6" t="n"/>
-      <c r="D41" s="16" t="n"/>
+      <c r="D41" s="18" t="n"/>
       <c r="E41" s="6" t="n"/>
       <c r="F41" s="6" t="n"/>
-      <c r="G41" s="16" t="n"/>
+      <c r="G41" s="18" t="n"/>
       <c r="H41" s="6">
         <f>IF(G41="","",G41-TODAY())</f>
         <v/>
@@ -4981,10 +4994,10 @@
       <c r="A42" s="14" t="n"/>
       <c r="B42" s="14" t="n"/>
       <c r="C42" s="14" t="n"/>
-      <c r="D42" s="15" t="n"/>
+      <c r="D42" s="17" t="n"/>
       <c r="E42" s="14" t="n"/>
       <c r="F42" s="14" t="n"/>
-      <c r="G42" s="15" t="n"/>
+      <c r="G42" s="17" t="n"/>
       <c r="H42" s="14">
         <f>IF(G42="","",G42-TODAY())</f>
         <v/>
@@ -4996,10 +5009,10 @@
       <c r="A43" s="6" t="n"/>
       <c r="B43" s="6" t="n"/>
       <c r="C43" s="6" t="n"/>
-      <c r="D43" s="16" t="n"/>
+      <c r="D43" s="18" t="n"/>
       <c r="E43" s="6" t="n"/>
       <c r="F43" s="6" t="n"/>
-      <c r="G43" s="16" t="n"/>
+      <c r="G43" s="18" t="n"/>
       <c r="H43" s="6">
         <f>IF(G43="","",G43-TODAY())</f>
         <v/>
@@ -5126,7 +5139,7 @@
           <t>EMP001</t>
         </is>
       </c>
-      <c r="F2" s="15" t="n">
+      <c r="F2" s="17" t="n">
         <v>46163</v>
       </c>
       <c r="G2" s="14" t="n"/>
@@ -5166,7 +5179,7 @@
           <t>EMP002</t>
         </is>
       </c>
-      <c r="F3" s="16" t="n">
+      <c r="F3" s="18" t="n">
         <v>46133</v>
       </c>
       <c r="G3" s="6" t="n"/>
@@ -5188,8 +5201,8 @@
       <c r="C4" s="14" t="n"/>
       <c r="D4" s="14" t="n"/>
       <c r="E4" s="14" t="n"/>
-      <c r="F4" s="15" t="n"/>
-      <c r="G4" s="15" t="n"/>
+      <c r="F4" s="17" t="n"/>
+      <c r="G4" s="17" t="n"/>
       <c r="H4" s="14" t="n"/>
       <c r="I4" s="14" t="n"/>
       <c r="J4" s="14" t="n"/>
@@ -5200,8 +5213,8 @@
       <c r="C5" s="6" t="n"/>
       <c r="D5" s="6" t="n"/>
       <c r="E5" s="6" t="n"/>
-      <c r="F5" s="16" t="n"/>
-      <c r="G5" s="16" t="n"/>
+      <c r="F5" s="18" t="n"/>
+      <c r="G5" s="18" t="n"/>
       <c r="H5" s="6" t="n"/>
       <c r="I5" s="6" t="n"/>
       <c r="J5" s="6" t="n"/>
@@ -5212,8 +5225,8 @@
       <c r="C6" s="14" t="n"/>
       <c r="D6" s="14" t="n"/>
       <c r="E6" s="14" t="n"/>
-      <c r="F6" s="15" t="n"/>
-      <c r="G6" s="15" t="n"/>
+      <c r="F6" s="17" t="n"/>
+      <c r="G6" s="17" t="n"/>
       <c r="H6" s="14" t="n"/>
       <c r="I6" s="14" t="n"/>
       <c r="J6" s="14" t="n"/>
@@ -5224,8 +5237,8 @@
       <c r="C7" s="6" t="n"/>
       <c r="D7" s="6" t="n"/>
       <c r="E7" s="6" t="n"/>
-      <c r="F7" s="16" t="n"/>
-      <c r="G7" s="16" t="n"/>
+      <c r="F7" s="18" t="n"/>
+      <c r="G7" s="18" t="n"/>
       <c r="H7" s="6" t="n"/>
       <c r="I7" s="6" t="n"/>
       <c r="J7" s="6" t="n"/>
@@ -5236,8 +5249,8 @@
       <c r="C8" s="14" t="n"/>
       <c r="D8" s="14" t="n"/>
       <c r="E8" s="14" t="n"/>
-      <c r="F8" s="15" t="n"/>
-      <c r="G8" s="15" t="n"/>
+      <c r="F8" s="17" t="n"/>
+      <c r="G8" s="17" t="n"/>
       <c r="H8" s="14" t="n"/>
       <c r="I8" s="14" t="n"/>
       <c r="J8" s="14" t="n"/>
@@ -5248,8 +5261,8 @@
       <c r="C9" s="6" t="n"/>
       <c r="D9" s="6" t="n"/>
       <c r="E9" s="6" t="n"/>
-      <c r="F9" s="16" t="n"/>
-      <c r="G9" s="16" t="n"/>
+      <c r="F9" s="18" t="n"/>
+      <c r="G9" s="18" t="n"/>
       <c r="H9" s="6" t="n"/>
       <c r="I9" s="6" t="n"/>
       <c r="J9" s="6" t="n"/>
@@ -5260,8 +5273,8 @@
       <c r="C10" s="14" t="n"/>
       <c r="D10" s="14" t="n"/>
       <c r="E10" s="14" t="n"/>
-      <c r="F10" s="15" t="n"/>
-      <c r="G10" s="15" t="n"/>
+      <c r="F10" s="17" t="n"/>
+      <c r="G10" s="17" t="n"/>
       <c r="H10" s="14" t="n"/>
       <c r="I10" s="14" t="n"/>
       <c r="J10" s="14" t="n"/>
@@ -5272,8 +5285,8 @@
       <c r="C11" s="6" t="n"/>
       <c r="D11" s="6" t="n"/>
       <c r="E11" s="6" t="n"/>
-      <c r="F11" s="16" t="n"/>
-      <c r="G11" s="16" t="n"/>
+      <c r="F11" s="18" t="n"/>
+      <c r="G11" s="18" t="n"/>
       <c r="H11" s="6" t="n"/>
       <c r="I11" s="6" t="n"/>
       <c r="J11" s="6" t="n"/>
@@ -5284,8 +5297,8 @@
       <c r="C12" s="14" t="n"/>
       <c r="D12" s="14" t="n"/>
       <c r="E12" s="14" t="n"/>
-      <c r="F12" s="15" t="n"/>
-      <c r="G12" s="15" t="n"/>
+      <c r="F12" s="17" t="n"/>
+      <c r="G12" s="17" t="n"/>
       <c r="H12" s="14" t="n"/>
       <c r="I12" s="14" t="n"/>
       <c r="J12" s="14" t="n"/>
@@ -5296,8 +5309,8 @@
       <c r="C13" s="6" t="n"/>
       <c r="D13" s="6" t="n"/>
       <c r="E13" s="6" t="n"/>
-      <c r="F13" s="16" t="n"/>
-      <c r="G13" s="16" t="n"/>
+      <c r="F13" s="18" t="n"/>
+      <c r="G13" s="18" t="n"/>
       <c r="H13" s="6" t="n"/>
       <c r="I13" s="6" t="n"/>
       <c r="J13" s="6" t="n"/>
@@ -5308,8 +5321,8 @@
       <c r="C14" s="14" t="n"/>
       <c r="D14" s="14" t="n"/>
       <c r="E14" s="14" t="n"/>
-      <c r="F14" s="15" t="n"/>
-      <c r="G14" s="15" t="n"/>
+      <c r="F14" s="17" t="n"/>
+      <c r="G14" s="17" t="n"/>
       <c r="H14" s="14" t="n"/>
       <c r="I14" s="14" t="n"/>
       <c r="J14" s="14" t="n"/>
@@ -5320,8 +5333,8 @@
       <c r="C15" s="6" t="n"/>
       <c r="D15" s="6" t="n"/>
       <c r="E15" s="6" t="n"/>
-      <c r="F15" s="16" t="n"/>
-      <c r="G15" s="16" t="n"/>
+      <c r="F15" s="18" t="n"/>
+      <c r="G15" s="18" t="n"/>
       <c r="H15" s="6" t="n"/>
       <c r="I15" s="6" t="n"/>
       <c r="J15" s="6" t="n"/>
@@ -5332,8 +5345,8 @@
       <c r="C16" s="14" t="n"/>
       <c r="D16" s="14" t="n"/>
       <c r="E16" s="14" t="n"/>
-      <c r="F16" s="15" t="n"/>
-      <c r="G16" s="15" t="n"/>
+      <c r="F16" s="17" t="n"/>
+      <c r="G16" s="17" t="n"/>
       <c r="H16" s="14" t="n"/>
       <c r="I16" s="14" t="n"/>
       <c r="J16" s="14" t="n"/>
@@ -5344,8 +5357,8 @@
       <c r="C17" s="6" t="n"/>
       <c r="D17" s="6" t="n"/>
       <c r="E17" s="6" t="n"/>
-      <c r="F17" s="16" t="n"/>
-      <c r="G17" s="16" t="n"/>
+      <c r="F17" s="18" t="n"/>
+      <c r="G17" s="18" t="n"/>
       <c r="H17" s="6" t="n"/>
       <c r="I17" s="6" t="n"/>
       <c r="J17" s="6" t="n"/>
@@ -5356,8 +5369,8 @@
       <c r="C18" s="14" t="n"/>
       <c r="D18" s="14" t="n"/>
       <c r="E18" s="14" t="n"/>
-      <c r="F18" s="15" t="n"/>
-      <c r="G18" s="15" t="n"/>
+      <c r="F18" s="17" t="n"/>
+      <c r="G18" s="17" t="n"/>
       <c r="H18" s="14" t="n"/>
       <c r="I18" s="14" t="n"/>
       <c r="J18" s="14" t="n"/>
@@ -5368,8 +5381,8 @@
       <c r="C19" s="6" t="n"/>
       <c r="D19" s="6" t="n"/>
       <c r="E19" s="6" t="n"/>
-      <c r="F19" s="16" t="n"/>
-      <c r="G19" s="16" t="n"/>
+      <c r="F19" s="18" t="n"/>
+      <c r="G19" s="18" t="n"/>
       <c r="H19" s="6" t="n"/>
       <c r="I19" s="6" t="n"/>
       <c r="J19" s="6" t="n"/>
@@ -5380,8 +5393,8 @@
       <c r="C20" s="14" t="n"/>
       <c r="D20" s="14" t="n"/>
       <c r="E20" s="14" t="n"/>
-      <c r="F20" s="15" t="n"/>
-      <c r="G20" s="15" t="n"/>
+      <c r="F20" s="17" t="n"/>
+      <c r="G20" s="17" t="n"/>
       <c r="H20" s="14" t="n"/>
       <c r="I20" s="14" t="n"/>
       <c r="J20" s="14" t="n"/>
@@ -5392,8 +5405,8 @@
       <c r="C21" s="6" t="n"/>
       <c r="D21" s="6" t="n"/>
       <c r="E21" s="6" t="n"/>
-      <c r="F21" s="16" t="n"/>
-      <c r="G21" s="16" t="n"/>
+      <c r="F21" s="18" t="n"/>
+      <c r="G21" s="18" t="n"/>
       <c r="H21" s="6" t="n"/>
       <c r="I21" s="6" t="n"/>
       <c r="J21" s="6" t="n"/>
@@ -5404,8 +5417,8 @@
       <c r="C22" s="14" t="n"/>
       <c r="D22" s="14" t="n"/>
       <c r="E22" s="14" t="n"/>
-      <c r="F22" s="15" t="n"/>
-      <c r="G22" s="15" t="n"/>
+      <c r="F22" s="17" t="n"/>
+      <c r="G22" s="17" t="n"/>
       <c r="H22" s="14" t="n"/>
       <c r="I22" s="14" t="n"/>
       <c r="J22" s="14" t="n"/>
@@ -5416,8 +5429,8 @@
       <c r="C23" s="6" t="n"/>
       <c r="D23" s="6" t="n"/>
       <c r="E23" s="6" t="n"/>
-      <c r="F23" s="16" t="n"/>
-      <c r="G23" s="16" t="n"/>
+      <c r="F23" s="18" t="n"/>
+      <c r="G23" s="18" t="n"/>
       <c r="H23" s="6" t="n"/>
       <c r="I23" s="6" t="n"/>
       <c r="J23" s="6" t="n"/>
@@ -5428,8 +5441,8 @@
       <c r="C24" s="14" t="n"/>
       <c r="D24" s="14" t="n"/>
       <c r="E24" s="14" t="n"/>
-      <c r="F24" s="15" t="n"/>
-      <c r="G24" s="15" t="n"/>
+      <c r="F24" s="17" t="n"/>
+      <c r="G24" s="17" t="n"/>
       <c r="H24" s="14" t="n"/>
       <c r="I24" s="14" t="n"/>
       <c r="J24" s="14" t="n"/>
@@ -5440,8 +5453,8 @@
       <c r="C25" s="6" t="n"/>
       <c r="D25" s="6" t="n"/>
       <c r="E25" s="6" t="n"/>
-      <c r="F25" s="16" t="n"/>
-      <c r="G25" s="16" t="n"/>
+      <c r="F25" s="18" t="n"/>
+      <c r="G25" s="18" t="n"/>
       <c r="H25" s="6" t="n"/>
       <c r="I25" s="6" t="n"/>
       <c r="J25" s="6" t="n"/>
@@ -5452,8 +5465,8 @@
       <c r="C26" s="14" t="n"/>
       <c r="D26" s="14" t="n"/>
       <c r="E26" s="14" t="n"/>
-      <c r="F26" s="15" t="n"/>
-      <c r="G26" s="15" t="n"/>
+      <c r="F26" s="17" t="n"/>
+      <c r="G26" s="17" t="n"/>
       <c r="H26" s="14" t="n"/>
       <c r="I26" s="14" t="n"/>
       <c r="J26" s="14" t="n"/>
@@ -5464,8 +5477,8 @@
       <c r="C27" s="6" t="n"/>
       <c r="D27" s="6" t="n"/>
       <c r="E27" s="6" t="n"/>
-      <c r="F27" s="16" t="n"/>
-      <c r="G27" s="16" t="n"/>
+      <c r="F27" s="18" t="n"/>
+      <c r="G27" s="18" t="n"/>
       <c r="H27" s="6" t="n"/>
       <c r="I27" s="6" t="n"/>
       <c r="J27" s="6" t="n"/>
@@ -5476,8 +5489,8 @@
       <c r="C28" s="14" t="n"/>
       <c r="D28" s="14" t="n"/>
       <c r="E28" s="14" t="n"/>
-      <c r="F28" s="15" t="n"/>
-      <c r="G28" s="15" t="n"/>
+      <c r="F28" s="17" t="n"/>
+      <c r="G28" s="17" t="n"/>
       <c r="H28" s="14" t="n"/>
       <c r="I28" s="14" t="n"/>
       <c r="J28" s="14" t="n"/>
@@ -5488,8 +5501,8 @@
       <c r="C29" s="6" t="n"/>
       <c r="D29" s="6" t="n"/>
       <c r="E29" s="6" t="n"/>
-      <c r="F29" s="16" t="n"/>
-      <c r="G29" s="16" t="n"/>
+      <c r="F29" s="18" t="n"/>
+      <c r="G29" s="18" t="n"/>
       <c r="H29" s="6" t="n"/>
       <c r="I29" s="6" t="n"/>
       <c r="J29" s="6" t="n"/>
@@ -5500,8 +5513,8 @@
       <c r="C30" s="14" t="n"/>
       <c r="D30" s="14" t="n"/>
       <c r="E30" s="14" t="n"/>
-      <c r="F30" s="15" t="n"/>
-      <c r="G30" s="15" t="n"/>
+      <c r="F30" s="17" t="n"/>
+      <c r="G30" s="17" t="n"/>
       <c r="H30" s="14" t="n"/>
       <c r="I30" s="14" t="n"/>
       <c r="J30" s="14" t="n"/>
@@ -5512,8 +5525,8 @@
       <c r="C31" s="6" t="n"/>
       <c r="D31" s="6" t="n"/>
       <c r="E31" s="6" t="n"/>
-      <c r="F31" s="16" t="n"/>
-      <c r="G31" s="16" t="n"/>
+      <c r="F31" s="18" t="n"/>
+      <c r="G31" s="18" t="n"/>
       <c r="H31" s="6" t="n"/>
       <c r="I31" s="6" t="n"/>
       <c r="J31" s="6" t="n"/>
@@ -5524,8 +5537,8 @@
       <c r="C32" s="14" t="n"/>
       <c r="D32" s="14" t="n"/>
       <c r="E32" s="14" t="n"/>
-      <c r="F32" s="15" t="n"/>
-      <c r="G32" s="15" t="n"/>
+      <c r="F32" s="17" t="n"/>
+      <c r="G32" s="17" t="n"/>
       <c r="H32" s="14" t="n"/>
       <c r="I32" s="14" t="n"/>
       <c r="J32" s="14" t="n"/>
@@ -5536,8 +5549,8 @@
       <c r="C33" s="6" t="n"/>
       <c r="D33" s="6" t="n"/>
       <c r="E33" s="6" t="n"/>
-      <c r="F33" s="16" t="n"/>
-      <c r="G33" s="16" t="n"/>
+      <c r="F33" s="18" t="n"/>
+      <c r="G33" s="18" t="n"/>
       <c r="H33" s="6" t="n"/>
       <c r="I33" s="6" t="n"/>
       <c r="J33" s="6" t="n"/>
@@ -5548,8 +5561,8 @@
       <c r="C34" s="14" t="n"/>
       <c r="D34" s="14" t="n"/>
       <c r="E34" s="14" t="n"/>
-      <c r="F34" s="15" t="n"/>
-      <c r="G34" s="15" t="n"/>
+      <c r="F34" s="17" t="n"/>
+      <c r="G34" s="17" t="n"/>
       <c r="H34" s="14" t="n"/>
       <c r="I34" s="14" t="n"/>
       <c r="J34" s="14" t="n"/>
@@ -5560,8 +5573,8 @@
       <c r="C35" s="6" t="n"/>
       <c r="D35" s="6" t="n"/>
       <c r="E35" s="6" t="n"/>
-      <c r="F35" s="16" t="n"/>
-      <c r="G35" s="16" t="n"/>
+      <c r="F35" s="18" t="n"/>
+      <c r="G35" s="18" t="n"/>
       <c r="H35" s="6" t="n"/>
       <c r="I35" s="6" t="n"/>
       <c r="J35" s="6" t="n"/>
@@ -5572,8 +5585,8 @@
       <c r="C36" s="14" t="n"/>
       <c r="D36" s="14" t="n"/>
       <c r="E36" s="14" t="n"/>
-      <c r="F36" s="15" t="n"/>
-      <c r="G36" s="15" t="n"/>
+      <c r="F36" s="17" t="n"/>
+      <c r="G36" s="17" t="n"/>
       <c r="H36" s="14" t="n"/>
       <c r="I36" s="14" t="n"/>
       <c r="J36" s="14" t="n"/>
@@ -5584,8 +5597,8 @@
       <c r="C37" s="6" t="n"/>
       <c r="D37" s="6" t="n"/>
       <c r="E37" s="6" t="n"/>
-      <c r="F37" s="16" t="n"/>
-      <c r="G37" s="16" t="n"/>
+      <c r="F37" s="18" t="n"/>
+      <c r="G37" s="18" t="n"/>
       <c r="H37" s="6" t="n"/>
       <c r="I37" s="6" t="n"/>
       <c r="J37" s="6" t="n"/>
@@ -5596,8 +5609,8 @@
       <c r="C38" s="14" t="n"/>
       <c r="D38" s="14" t="n"/>
       <c r="E38" s="14" t="n"/>
-      <c r="F38" s="15" t="n"/>
-      <c r="G38" s="15" t="n"/>
+      <c r="F38" s="17" t="n"/>
+      <c r="G38" s="17" t="n"/>
       <c r="H38" s="14" t="n"/>
       <c r="I38" s="14" t="n"/>
       <c r="J38" s="14" t="n"/>
@@ -5608,8 +5621,8 @@
       <c r="C39" s="6" t="n"/>
       <c r="D39" s="6" t="n"/>
       <c r="E39" s="6" t="n"/>
-      <c r="F39" s="16" t="n"/>
-      <c r="G39" s="16" t="n"/>
+      <c r="F39" s="18" t="n"/>
+      <c r="G39" s="18" t="n"/>
       <c r="H39" s="6" t="n"/>
       <c r="I39" s="6" t="n"/>
       <c r="J39" s="6" t="n"/>
@@ -5620,8 +5633,8 @@
       <c r="C40" s="14" t="n"/>
       <c r="D40" s="14" t="n"/>
       <c r="E40" s="14" t="n"/>
-      <c r="F40" s="15" t="n"/>
-      <c r="G40" s="15" t="n"/>
+      <c r="F40" s="17" t="n"/>
+      <c r="G40" s="17" t="n"/>
       <c r="H40" s="14" t="n"/>
       <c r="I40" s="14" t="n"/>
       <c r="J40" s="14" t="n"/>
@@ -5632,8 +5645,8 @@
       <c r="C41" s="6" t="n"/>
       <c r="D41" s="6" t="n"/>
       <c r="E41" s="6" t="n"/>
-      <c r="F41" s="16" t="n"/>
-      <c r="G41" s="16" t="n"/>
+      <c r="F41" s="18" t="n"/>
+      <c r="G41" s="18" t="n"/>
       <c r="H41" s="6" t="n"/>
       <c r="I41" s="6" t="n"/>
       <c r="J41" s="6" t="n"/>
@@ -5644,8 +5657,8 @@
       <c r="C42" s="14" t="n"/>
       <c r="D42" s="14" t="n"/>
       <c r="E42" s="14" t="n"/>
-      <c r="F42" s="15" t="n"/>
-      <c r="G42" s="15" t="n"/>
+      <c r="F42" s="17" t="n"/>
+      <c r="G42" s="17" t="n"/>
       <c r="H42" s="14" t="n"/>
       <c r="I42" s="14" t="n"/>
       <c r="J42" s="14" t="n"/>
@@ -5656,8 +5669,8 @@
       <c r="C43" s="6" t="n"/>
       <c r="D43" s="6" t="n"/>
       <c r="E43" s="6" t="n"/>
-      <c r="F43" s="16" t="n"/>
-      <c r="G43" s="16" t="n"/>
+      <c r="F43" s="18" t="n"/>
+      <c r="G43" s="18" t="n"/>
       <c r="H43" s="6" t="n"/>
       <c r="I43" s="6" t="n"/>
       <c r="J43" s="6" t="n"/>

</xml_diff>

<commit_message>
Add employee Aneesh Kumar (EMP003) to Employee List
</commit_message>
<xml_diff>
--- a/Compliance_Management_Tracker.xlsx
+++ b/Compliance_Management_Tracker.xlsx
@@ -3047,11 +3047,23 @@
       <c r="J3" s="6" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="14" t="n"/>
-      <c r="B4" s="14" t="n"/>
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>EMP003</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>Aneesh Kumar</t>
+        </is>
+      </c>
       <c r="C4" s="14" t="n"/>
       <c r="D4" s="14" t="n"/>
-      <c r="E4" s="14" t="n"/>
+      <c r="E4" s="14" t="inlineStr">
+        <is>
+          <t>6306177706</t>
+        </is>
+      </c>
       <c r="F4" s="14" t="n"/>
       <c r="G4" s="14" t="n"/>
       <c r="H4" s="17" t="n"/>

</xml_diff>